<commit_message>
Add data for 2026-02-23
</commit_message>
<xml_diff>
--- a/output/index-crime-full-year.xlsx
+++ b/output/index-crime-full-year.xlsx
@@ -913,7 +913,7 @@
         <v>6579</v>
       </c>
       <c r="M2">
-        <v>758</v>
+        <v>766</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -954,7 +954,7 @@
         <v>7108</v>
       </c>
       <c r="M3">
-        <v>828</v>
+        <v>848</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -992,10 +992,10 @@
         <v>481</v>
       </c>
       <c r="L4">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="M4">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1033,10 +1033,10 @@
         <v>7656</v>
       </c>
       <c r="L5">
-        <v>6184</v>
+        <v>6185</v>
       </c>
       <c r="M5">
-        <v>669</v>
+        <v>684</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1065,7 +1065,7 @@
         <v>1774</v>
       </c>
       <c r="I6">
-        <v>1850</v>
+        <v>1851</v>
       </c>
       <c r="J6">
         <v>1892</v>
@@ -1074,10 +1074,10 @@
         <v>1802</v>
       </c>
       <c r="L6">
-        <v>1808</v>
+        <v>1809</v>
       </c>
       <c r="M6">
-        <v>231</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1156,10 +1156,10 @@
         <v>21711</v>
       </c>
       <c r="L8">
-        <v>17229</v>
+        <v>17230</v>
       </c>
       <c r="M8">
-        <v>2369</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1200,7 +1200,7 @@
         <v>5817</v>
       </c>
       <c r="M9">
-        <v>624</v>
+        <v>627</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1241,7 +1241,7 @@
         <v>58553</v>
       </c>
       <c r="M10">
-        <v>6878</v>
+        <v>6979</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1270,7 +1270,7 @@
         <v>84710</v>
       </c>
       <c r="I11">
-        <v>110708</v>
+        <v>110709</v>
       </c>
       <c r="J11">
         <v>124134</v>
@@ -1279,10 +1279,10 @@
         <v>118748</v>
       </c>
       <c r="L11">
-        <v>104074</v>
+        <v>104078</v>
       </c>
       <c r="M11">
-        <v>12444</v>
+        <v>12643</v>
       </c>
     </row>
   </sheetData>
@@ -1635,7 +1635,7 @@
         <v>183</v>
       </c>
       <c r="M8">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1717,7 +1717,7 @@
         <v>685</v>
       </c>
       <c r="M10">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1758,7 +1758,7 @@
         <v>1413</v>
       </c>
       <c r="M11">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -2664,7 +2664,7 @@
         <v>72</v>
       </c>
       <c r="M2">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2784,7 +2784,7 @@
         <v>96</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2901,7 +2901,7 @@
         <v>223</v>
       </c>
       <c r="M8">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2983,7 +2983,7 @@
         <v>1212</v>
       </c>
       <c r="M10">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3024,7 +3024,7 @@
         <v>1774</v>
       </c>
       <c r="M11">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -3131,7 +3131,7 @@
         <v>438</v>
       </c>
       <c r="M2">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3172,7 +3172,7 @@
         <v>504</v>
       </c>
       <c r="M3">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3295,7 +3295,7 @@
         <v>106</v>
       </c>
       <c r="M6">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3377,7 +3377,7 @@
         <v>776</v>
       </c>
       <c r="M8">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3459,7 +3459,7 @@
         <v>1974</v>
       </c>
       <c r="M10">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3500,7 +3500,7 @@
         <v>4436</v>
       </c>
       <c r="M11">
-        <v>500</v>
+        <v>509</v>
       </c>
     </row>
   </sheetData>
@@ -3712,7 +3712,7 @@
         <v>15</v>
       </c>
       <c r="M5">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3940,7 +3940,7 @@
         <v>302</v>
       </c>
       <c r="M11">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -4088,7 +4088,7 @@
         <v>47</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4287,7 +4287,7 @@
         <v>105</v>
       </c>
       <c r="M8">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4410,7 +4410,7 @@
         <v>740</v>
       </c>
       <c r="M11">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -4736,7 +4736,7 @@
         <v>119</v>
       </c>
       <c r="M8">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4859,7 +4859,7 @@
         <v>345</v>
       </c>
       <c r="M11">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -5291,7 +5291,7 @@
         <v>495</v>
       </c>
       <c r="M10">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5332,7 +5332,7 @@
         <v>1490</v>
       </c>
       <c r="M11">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -5480,7 +5480,7 @@
         <v>343</v>
       </c>
       <c r="M3">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5562,7 +5562,7 @@
         <v>125</v>
       </c>
       <c r="M5">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -5685,7 +5685,7 @@
         <v>461</v>
       </c>
       <c r="M8">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5767,7 +5767,7 @@
         <v>875</v>
       </c>
       <c r="M10">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5808,7 +5808,7 @@
         <v>2444</v>
       </c>
       <c r="M11">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -6240,7 +6240,7 @@
         <v>864</v>
       </c>
       <c r="M10">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6281,7 +6281,7 @@
         <v>2096</v>
       </c>
       <c r="M11">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -6388,7 +6388,7 @@
         <v>929</v>
       </c>
       <c r="M2">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6552,7 +6552,7 @@
         <v>780</v>
       </c>
       <c r="M6">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -6593,7 +6593,7 @@
         <v>2419</v>
       </c>
       <c r="M7">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6634,7 +6634,7 @@
         <v>4436</v>
       </c>
       <c r="M8">
-        <v>500</v>
+        <v>509</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6675,7 +6675,7 @@
         <v>448</v>
       </c>
       <c r="M9">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6716,7 +6716,7 @@
         <v>1155</v>
       </c>
       <c r="M10">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6757,7 +6757,7 @@
         <v>1780</v>
       </c>
       <c r="M11">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6798,7 +6798,7 @@
         <v>415</v>
       </c>
       <c r="M12">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -6880,7 +6880,7 @@
         <v>730</v>
       </c>
       <c r="M14">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -6962,7 +6962,7 @@
         <v>751</v>
       </c>
       <c r="M16">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7044,7 +7044,7 @@
         <v>644</v>
       </c>
       <c r="M18">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -7085,7 +7085,7 @@
         <v>2348</v>
       </c>
       <c r="M19">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -7249,7 +7249,7 @@
         <v>1351</v>
       </c>
       <c r="M23">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -7290,7 +7290,7 @@
         <v>533</v>
       </c>
       <c r="M24">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -7413,7 +7413,7 @@
         <v>1244</v>
       </c>
       <c r="M27">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -7483,7 +7483,7 @@
         <v>3519</v>
       </c>
       <c r="I29">
-        <v>3980</v>
+        <v>3981</v>
       </c>
       <c r="J29">
         <v>4175</v>
@@ -7492,10 +7492,10 @@
         <v>3878</v>
       </c>
       <c r="L29">
-        <v>3375</v>
+        <v>3376</v>
       </c>
       <c r="M29">
-        <v>412</v>
+        <v>417</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7577,7 +7577,7 @@
         <v>1014</v>
       </c>
       <c r="M31">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -7659,7 +7659,7 @@
         <v>2444</v>
       </c>
       <c r="M33">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -7700,7 +7700,7 @@
         <v>706</v>
       </c>
       <c r="M34">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -7782,7 +7782,7 @@
         <v>1431</v>
       </c>
       <c r="M36">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7823,7 +7823,7 @@
         <v>2341</v>
       </c>
       <c r="M37">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -8025,10 +8025,10 @@
         <v>3266</v>
       </c>
       <c r="L42">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="M42">
-        <v>313</v>
+        <v>322</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -8069,7 +8069,7 @@
         <v>1468</v>
       </c>
       <c r="M43">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -8110,7 +8110,7 @@
         <v>972</v>
       </c>
       <c r="M44">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -8192,7 +8192,7 @@
         <v>302</v>
       </c>
       <c r="M46">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -8233,7 +8233,7 @@
         <v>945</v>
       </c>
       <c r="M47">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -8274,7 +8274,7 @@
         <v>2778</v>
       </c>
       <c r="M48">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -8312,10 +8312,10 @@
         <v>2190</v>
       </c>
       <c r="L49">
-        <v>1781</v>
+        <v>1782</v>
       </c>
       <c r="M49">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -8397,7 +8397,7 @@
         <v>1453</v>
       </c>
       <c r="M51">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -8438,7 +8438,7 @@
         <v>1413</v>
       </c>
       <c r="M52">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -8479,7 +8479,7 @@
         <v>1774</v>
       </c>
       <c r="M53">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -8520,7 +8520,7 @@
         <v>3846</v>
       </c>
       <c r="M54">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -8561,7 +8561,7 @@
         <v>1081</v>
       </c>
       <c r="M55">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -8602,7 +8602,7 @@
         <v>621</v>
       </c>
       <c r="M56">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -8643,7 +8643,7 @@
         <v>470</v>
       </c>
       <c r="M57">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -8725,7 +8725,7 @@
         <v>299</v>
       </c>
       <c r="M59">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -8766,7 +8766,7 @@
         <v>740</v>
       </c>
       <c r="M60">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -8886,10 +8886,10 @@
         <v>867</v>
       </c>
       <c r="L63">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="M63">
-        <v>53</v>
+        <v>64</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -8930,7 +8930,7 @@
         <v>949</v>
       </c>
       <c r="M64">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -8968,10 +8968,10 @@
         <v>1684</v>
       </c>
       <c r="L65">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="M65">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -9012,7 +9012,7 @@
         <v>602</v>
       </c>
       <c r="M66">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -9053,7 +9053,7 @@
         <v>1927</v>
       </c>
       <c r="M67">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -9094,7 +9094,7 @@
         <v>500</v>
       </c>
       <c r="M68">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -9176,7 +9176,7 @@
         <v>656</v>
       </c>
       <c r="M70">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -9217,7 +9217,7 @@
         <v>345</v>
       </c>
       <c r="M71">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="72" spans="1:13">
@@ -9299,7 +9299,7 @@
         <v>1356</v>
       </c>
       <c r="M73">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -9381,7 +9381,7 @@
         <v>428</v>
       </c>
       <c r="M75">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -9422,7 +9422,7 @@
         <v>3358</v>
       </c>
       <c r="M76">
-        <v>378</v>
+        <v>385</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -9504,7 +9504,7 @@
         <v>1586</v>
       </c>
       <c r="M78">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -9545,7 +9545,7 @@
         <v>2096</v>
       </c>
       <c r="M79">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -9586,7 +9586,7 @@
         <v>477</v>
       </c>
       <c r="M80">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -9627,7 +9627,7 @@
         <v>186</v>
       </c>
       <c r="M81">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -9709,7 +9709,7 @@
         <v>1490</v>
       </c>
       <c r="M83">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -9750,7 +9750,7 @@
         <v>842</v>
       </c>
       <c r="M84">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="85" spans="1:13">
@@ -9788,10 +9788,10 @@
         <v>3840</v>
       </c>
       <c r="L85">
-        <v>3419</v>
+        <v>3420</v>
       </c>
       <c r="M85">
-        <v>404</v>
+        <v>410</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -9829,10 +9829,10 @@
         <v>1010</v>
       </c>
       <c r="L86">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="M86">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -9873,7 +9873,7 @@
         <v>440</v>
       </c>
       <c r="M87">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -9914,7 +9914,7 @@
         <v>880</v>
       </c>
       <c r="M88">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -9955,7 +9955,7 @@
         <v>2047</v>
       </c>
       <c r="M89">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -9996,7 +9996,7 @@
         <v>1095</v>
       </c>
       <c r="M90">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -10037,7 +10037,7 @@
         <v>971</v>
       </c>
       <c r="M91">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -10078,7 +10078,7 @@
         <v>318</v>
       </c>
       <c r="M92">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="93" spans="1:13">
@@ -10119,7 +10119,7 @@
         <v>810</v>
       </c>
       <c r="M93">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="94" spans="1:13">
@@ -10160,7 +10160,7 @@
         <v>2677</v>
       </c>
       <c r="M94">
-        <v>354</v>
+        <v>358</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -10198,10 +10198,10 @@
         <v>1446</v>
       </c>
       <c r="L95">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="M95">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -10242,7 +10242,7 @@
         <v>1361</v>
       </c>
       <c r="M96">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -10365,7 +10365,7 @@
         <v>1514</v>
       </c>
       <c r="M99">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -10435,7 +10435,7 @@
         <v>84710</v>
       </c>
       <c r="I101">
-        <v>110708</v>
+        <v>110709</v>
       </c>
       <c r="J101">
         <v>124134</v>
@@ -10444,10 +10444,10 @@
         <v>118748</v>
       </c>
       <c r="L101">
-        <v>104074</v>
+        <v>104078</v>
       </c>
       <c r="M101">
-        <v>12444</v>
+        <v>12643</v>
       </c>
     </row>
   </sheetData>
@@ -10697,7 +10697,7 @@
         <v>28</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -10875,7 +10875,7 @@
         <v>64</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -10995,7 +10995,7 @@
         <v>428</v>
       </c>
       <c r="M11">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -11764,7 +11764,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11887,7 +11887,7 @@
         <v>949</v>
       </c>
       <c r="M11">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -11994,7 +11994,7 @@
         <v>107</v>
       </c>
       <c r="M2">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -12117,7 +12117,7 @@
         <v>147</v>
       </c>
       <c r="M5">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -12240,7 +12240,7 @@
         <v>285</v>
       </c>
       <c r="M8">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -12319,7 +12319,7 @@
         <v>545</v>
       </c>
       <c r="L10">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="M10">
         <v>50</v>
@@ -12360,10 +12360,10 @@
         <v>1446</v>
       </c>
       <c r="L11">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="M11">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -12593,7 +12593,7 @@
         <v>172</v>
       </c>
       <c r="M5">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -12713,7 +12713,7 @@
         <v>417</v>
       </c>
       <c r="M8">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -12795,7 +12795,7 @@
         <v>900</v>
       </c>
       <c r="M10">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12836,7 +12836,7 @@
         <v>2341</v>
       </c>
       <c r="M11">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -12981,7 +12981,7 @@
         <v>151</v>
       </c>
       <c r="L3">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M3">
         <v>20</v>
@@ -13186,7 +13186,7 @@
         <v>233</v>
       </c>
       <c r="M8">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13265,10 +13265,10 @@
         <v>637</v>
       </c>
       <c r="L10">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="M10">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13306,10 +13306,10 @@
         <v>1684</v>
       </c>
       <c r="L11">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="M11">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -13530,7 +13530,7 @@
         <v>105</v>
       </c>
       <c r="M5">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13726,7 +13726,7 @@
         <v>818</v>
       </c>
       <c r="M10">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13767,7 +13767,7 @@
         <v>1244</v>
       </c>
       <c r="M11">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -13915,7 +13915,7 @@
         <v>150</v>
       </c>
       <c r="M3">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -14202,7 +14202,7 @@
         <v>753</v>
       </c>
       <c r="M10">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -14243,7 +14243,7 @@
         <v>1514</v>
       </c>
       <c r="M11">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -15133,7 +15133,7 @@
         <v>606</v>
       </c>
       <c r="M10">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15174,7 +15174,7 @@
         <v>1014</v>
       </c>
       <c r="M11">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -15398,7 +15398,7 @@
         <v>76</v>
       </c>
       <c r="M5">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -15632,7 +15632,7 @@
         <v>730</v>
       </c>
       <c r="M11">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -15780,7 +15780,7 @@
         <v>295</v>
       </c>
       <c r="M3">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -15985,7 +15985,7 @@
         <v>322</v>
       </c>
       <c r="M8">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16026,7 +16026,7 @@
         <v>177</v>
       </c>
       <c r="M9">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -16067,7 +16067,7 @@
         <v>739</v>
       </c>
       <c r="M10">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16108,7 +16108,7 @@
         <v>1927</v>
       </c>
       <c r="M11">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -16455,7 +16455,7 @@
         <v>194</v>
       </c>
       <c r="M8">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16578,7 +16578,7 @@
         <v>842</v>
       </c>
       <c r="M11">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -16910,7 +16910,7 @@
         <v>358</v>
       </c>
       <c r="M8">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16951,7 +16951,7 @@
         <v>95</v>
       </c>
       <c r="M9">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -16992,7 +16992,7 @@
         <v>1963</v>
       </c>
       <c r="M10">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17033,7 +17033,7 @@
         <v>2677</v>
       </c>
       <c r="M11">
-        <v>354</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -17377,7 +17377,7 @@
         <v>211</v>
       </c>
       <c r="M8">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17459,7 +17459,7 @@
         <v>2712</v>
       </c>
       <c r="M10">
-        <v>302</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17500,7 +17500,7 @@
         <v>3358</v>
       </c>
       <c r="M11">
-        <v>378</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -17902,7 +17902,7 @@
         <v>304</v>
       </c>
       <c r="M10">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17943,7 +17943,7 @@
         <v>440</v>
       </c>
       <c r="M11">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -18961,6 +18961,9 @@
       <c r="L3">
         <v>7</v>
       </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
@@ -19201,7 +19204,7 @@
         <v>592</v>
       </c>
       <c r="M10">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19242,7 +19245,7 @@
         <v>751</v>
       </c>
       <c r="M11">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -19390,7 +19393,7 @@
         <v>17</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -19466,7 +19469,7 @@
         <v>124</v>
       </c>
       <c r="M5">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -19650,10 +19653,10 @@
         <v>1651</v>
       </c>
       <c r="L10">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="M10">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19691,10 +19694,10 @@
         <v>2190</v>
       </c>
       <c r="L11">
-        <v>1781</v>
+        <v>1782</v>
       </c>
       <c r="M11">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -20514,7 +20517,7 @@
         <v>252</v>
       </c>
       <c r="M8">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20596,7 +20599,7 @@
         <v>763</v>
       </c>
       <c r="M10">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20637,7 +20640,7 @@
         <v>1361</v>
       </c>
       <c r="M11">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -20785,7 +20788,7 @@
         <v>76</v>
       </c>
       <c r="M3">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -20864,7 +20867,7 @@
         <v>80</v>
       </c>
       <c r="M5">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -20987,7 +20990,7 @@
         <v>183</v>
       </c>
       <c r="M8">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21028,7 +21031,7 @@
         <v>62</v>
       </c>
       <c r="M9">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -21110,7 +21113,7 @@
         <v>1081</v>
       </c>
       <c r="M11">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -21542,7 +21545,7 @@
         <v>2938</v>
       </c>
       <c r="M10">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21583,7 +21586,7 @@
         <v>3846</v>
       </c>
       <c r="M11">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
   </sheetData>
@@ -21851,7 +21854,7 @@
         <v>17</v>
       </c>
       <c r="M6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -22012,7 +22015,7 @@
         <v>904</v>
       </c>
       <c r="M10">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22053,7 +22056,7 @@
         <v>1356</v>
       </c>
       <c r="M11">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -22201,7 +22204,7 @@
         <v>468</v>
       </c>
       <c r="M3">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -22312,7 +22315,7 @@
         <v>69</v>
       </c>
       <c r="I6">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="J6">
         <v>84</v>
@@ -22324,7 +22327,7 @@
         <v>67</v>
       </c>
       <c r="M6">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -22406,7 +22409,7 @@
         <v>644</v>
       </c>
       <c r="M8">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22485,10 +22488,10 @@
         <v>1294</v>
       </c>
       <c r="L10">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="M10">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22517,7 +22520,7 @@
         <v>3519</v>
       </c>
       <c r="I11">
-        <v>3980</v>
+        <v>3981</v>
       </c>
       <c r="J11">
         <v>4175</v>
@@ -22526,10 +22529,10 @@
         <v>3878</v>
       </c>
       <c r="L11">
-        <v>3375</v>
+        <v>3376</v>
       </c>
       <c r="M11">
-        <v>412</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -22750,7 +22753,7 @@
         <v>233</v>
       </c>
       <c r="L5">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="M5">
         <v>15</v>
@@ -22864,7 +22867,7 @@
         <v>253</v>
       </c>
       <c r="M8">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22943,10 +22946,10 @@
         <v>2259</v>
       </c>
       <c r="L10">
-        <v>2039</v>
+        <v>2038</v>
       </c>
       <c r="M10">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22987,7 +22990,7 @@
         <v>2778</v>
       </c>
       <c r="M11">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -23135,7 +23138,7 @@
         <v>181</v>
       </c>
       <c r="M3">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -23340,7 +23343,7 @@
         <v>412</v>
       </c>
       <c r="M8">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23422,7 +23425,7 @@
         <v>1136</v>
       </c>
       <c r="M10">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23463,7 +23466,7 @@
         <v>2348</v>
       </c>
       <c r="M11">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -23859,7 +23862,7 @@
         <v>383</v>
       </c>
       <c r="M10">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23900,7 +23903,7 @@
         <v>602</v>
       </c>
       <c r="M11">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -24241,7 +24244,7 @@
         <v>150</v>
       </c>
       <c r="M8">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24323,7 +24326,7 @@
         <v>604</v>
       </c>
       <c r="M10">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24364,7 +24367,7 @@
         <v>972</v>
       </c>
       <c r="M11">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -24471,7 +24474,7 @@
         <v>187</v>
       </c>
       <c r="M2">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -24512,7 +24515,7 @@
         <v>235</v>
       </c>
       <c r="M3">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -24594,7 +24597,7 @@
         <v>136</v>
       </c>
       <c r="M5">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -24632,7 +24635,7 @@
         <v>48</v>
       </c>
       <c r="L6">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M6">
         <v>8</v>
@@ -24717,7 +24720,7 @@
         <v>498</v>
       </c>
       <c r="M8">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24799,7 +24802,7 @@
         <v>1167</v>
       </c>
       <c r="M10">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24837,10 +24840,10 @@
         <v>3266</v>
       </c>
       <c r="L11">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="M11">
-        <v>313</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -25721,7 +25724,7 @@
         <v>941</v>
       </c>
       <c r="M10">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25762,7 +25765,7 @@
         <v>2419</v>
       </c>
       <c r="M11">
-        <v>301</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -25910,7 +25913,7 @@
         <v>51</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -26188,7 +26191,7 @@
         <v>320</v>
       </c>
       <c r="M10">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26229,7 +26232,7 @@
         <v>780</v>
       </c>
       <c r="M11">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -26917,7 +26920,7 @@
         <v>78</v>
       </c>
       <c r="M5">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -27160,7 +27163,7 @@
         <v>1431</v>
       </c>
       <c r="M11">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -27791,7 +27794,7 @@
         <v>61</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -27990,7 +27993,7 @@
         <v>826</v>
       </c>
       <c r="M10">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28031,7 +28034,7 @@
         <v>1155</v>
       </c>
       <c r="M11">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -28421,10 +28424,10 @@
         <v>724</v>
       </c>
       <c r="L10">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="M10">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28462,10 +28465,10 @@
         <v>1010</v>
       </c>
       <c r="L11">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="M11">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -28572,7 +28575,7 @@
         <v>75</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -28733,7 +28736,7 @@
         <v>33</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -28812,7 +28815,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -28894,7 +28897,7 @@
         <v>979</v>
       </c>
       <c r="M10">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28935,7 +28938,7 @@
         <v>1586</v>
       </c>
       <c r="M11">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -29337,7 +29340,7 @@
         <v>329</v>
       </c>
       <c r="M10">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29378,7 +29381,7 @@
         <v>500</v>
       </c>
       <c r="M11">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -29526,7 +29529,7 @@
         <v>21</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -29789,7 +29792,7 @@
         <v>307</v>
       </c>
       <c r="M10">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29830,7 +29833,7 @@
         <v>533</v>
       </c>
       <c r="M11">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -30413,7 +30416,7 @@
         <v>133</v>
       </c>
       <c r="M2">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -30454,7 +30457,7 @@
         <v>99</v>
       </c>
       <c r="M3">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -30653,7 +30656,7 @@
         <v>284</v>
       </c>
       <c r="M8">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -30735,7 +30738,7 @@
         <v>1042</v>
       </c>
       <c r="M10">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30776,7 +30779,7 @@
         <v>1780</v>
       </c>
       <c r="M11">
-        <v>236</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -31199,7 +31202,7 @@
         <v>722</v>
       </c>
       <c r="M10">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31240,7 +31243,7 @@
         <v>1351</v>
       </c>
       <c r="M11">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -31388,7 +31391,7 @@
         <v>132</v>
       </c>
       <c r="M3">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -31593,7 +31596,7 @@
         <v>250</v>
       </c>
       <c r="M8">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -31675,7 +31678,7 @@
         <v>380</v>
       </c>
       <c r="M10">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31716,7 +31719,7 @@
         <v>971</v>
       </c>
       <c r="M11">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -32145,7 +32148,7 @@
         <v>818</v>
       </c>
       <c r="M10">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32186,7 +32189,7 @@
         <v>1453</v>
       </c>
       <c r="M11">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -33416,7 +33419,7 @@
         <v>195</v>
       </c>
       <c r="M8">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -33539,7 +33542,7 @@
         <v>945</v>
       </c>
       <c r="M11">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -33886,7 +33889,7 @@
         <v>294</v>
       </c>
       <c r="M8">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -33968,7 +33971,7 @@
         <v>483</v>
       </c>
       <c r="M10">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34009,7 +34012,7 @@
         <v>1095</v>
       </c>
       <c r="M11">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -34884,7 +34887,7 @@
         <v>490</v>
       </c>
       <c r="M10">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34925,7 +34928,7 @@
         <v>810</v>
       </c>
       <c r="M11">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -35351,7 +35354,7 @@
         <v>267</v>
       </c>
       <c r="M10">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35392,7 +35395,7 @@
         <v>644</v>
       </c>
       <c r="M11">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -35540,7 +35543,7 @@
         <v>17</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -35776,7 +35779,7 @@
         <v>530</v>
       </c>
       <c r="M10">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35817,7 +35820,7 @@
         <v>656</v>
       </c>
       <c r="M11">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -36653,7 +36656,7 @@
         <v>585</v>
       </c>
       <c r="M10">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36694,7 +36697,7 @@
         <v>621</v>
       </c>
       <c r="M11">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -37566,7 +37569,7 @@
         <v>534</v>
       </c>
       <c r="M10">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -37607,7 +37610,7 @@
         <v>929</v>
       </c>
       <c r="M11">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -38306,7 +38309,7 @@
         <v>27</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -38455,7 +38458,7 @@
         <v>1039</v>
       </c>
       <c r="M10">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38496,7 +38499,7 @@
         <v>1468</v>
       </c>
       <c r="M11">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -39527,7 +39530,7 @@
         <v>17</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -39760,7 +39763,7 @@
         <v>372</v>
       </c>
       <c r="M10">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -39801,7 +39804,7 @@
         <v>477</v>
       </c>
       <c r="M11">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -40028,7 +40031,7 @@
         <v>52</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -40227,7 +40230,7 @@
         <v>389</v>
       </c>
       <c r="M10">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40268,7 +40271,7 @@
         <v>706</v>
       </c>
       <c r="M11">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -40697,7 +40700,7 @@
         <v>1436</v>
       </c>
       <c r="M10">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40738,7 +40741,7 @@
         <v>2047</v>
       </c>
       <c r="M11">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -43297,7 +43300,7 @@
         <v>29</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -43654,7 +43657,7 @@
         <v>318</v>
       </c>
       <c r="M11">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -44906,7 +44909,7 @@
         <v>171</v>
       </c>
       <c r="M10">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -44947,7 +44950,7 @@
         <v>448</v>
       </c>
       <c r="M11">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -45133,7 +45136,10 @@
         <v>20</v>
       </c>
       <c r="L4">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -45174,7 +45180,7 @@
         <v>309</v>
       </c>
       <c r="M5">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -45215,7 +45221,7 @@
         <v>65</v>
       </c>
       <c r="M6">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -45297,7 +45303,7 @@
         <v>642</v>
       </c>
       <c r="M8">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45417,10 +45423,10 @@
         <v>3840</v>
       </c>
       <c r="L11">
-        <v>3419</v>
+        <v>3420</v>
       </c>
       <c r="M11">
-        <v>404</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -45734,7 +45740,7 @@
         <v>65</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45857,7 +45863,7 @@
         <v>299</v>
       </c>
       <c r="M11">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -46653,7 +46659,7 @@
         <v>296</v>
       </c>
       <c r="M10">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -46694,7 +46700,7 @@
         <v>470</v>
       </c>
       <c r="M11">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -47038,7 +47044,7 @@
         <v>183</v>
       </c>
       <c r="M8">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -47161,7 +47167,7 @@
         <v>880</v>
       </c>
       <c r="M11">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -48099,7 +48105,7 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -48154,7 +48160,7 @@
         <v>24</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -48355,7 +48361,7 @@
         <v>186</v>
       </c>
       <c r="M11">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -48837,7 +48843,7 @@
         <v>14</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -49170,7 +49176,7 @@
         <v>415</v>
       </c>
       <c r="M11">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-02-25
</commit_message>
<xml_diff>
--- a/output/index-crime-full-year.xlsx
+++ b/output/index-crime-full-year.xlsx
@@ -913,7 +913,7 @@
         <v>6579</v>
       </c>
       <c r="M2">
-        <v>770</v>
+        <v>784</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -951,10 +951,10 @@
         <v>8180</v>
       </c>
       <c r="L3">
-        <v>7108</v>
+        <v>7109</v>
       </c>
       <c r="M3">
-        <v>858</v>
+        <v>871</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1036,7 +1036,7 @@
         <v>6184</v>
       </c>
       <c r="M5">
-        <v>692</v>
+        <v>708</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1071,13 +1071,13 @@
         <v>1892</v>
       </c>
       <c r="K6">
-        <v>1801</v>
+        <v>1803</v>
       </c>
       <c r="L6">
-        <v>1807</v>
+        <v>1808</v>
       </c>
       <c r="M6">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1118,7 +1118,7 @@
         <v>424</v>
       </c>
       <c r="M7">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1156,10 +1156,10 @@
         <v>21711</v>
       </c>
       <c r="L8">
-        <v>17229</v>
+        <v>17231</v>
       </c>
       <c r="M8">
-        <v>2448</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1200,7 +1200,7 @@
         <v>5817</v>
       </c>
       <c r="M9">
-        <v>642</v>
+        <v>647</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1241,7 +1241,7 @@
         <v>58556</v>
       </c>
       <c r="M10">
-        <v>7101</v>
+        <v>7251</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1276,13 +1276,13 @@
         <v>124135</v>
       </c>
       <c r="K11">
-        <v>118747</v>
+        <v>118749</v>
       </c>
       <c r="L11">
-        <v>104077</v>
+        <v>104081</v>
       </c>
       <c r="M11">
-        <v>12846</v>
+        <v>13086</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1389,7 @@
         <v>146</v>
       </c>
       <c r="M2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1430,7 +1430,7 @@
         <v>142</v>
       </c>
       <c r="M3">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1509,7 +1509,7 @@
         <v>52</v>
       </c>
       <c r="L5">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="M5">
         <v>6</v>
@@ -1717,7 +1717,7 @@
         <v>685</v>
       </c>
       <c r="M10">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1755,10 +1755,10 @@
         <v>1848</v>
       </c>
       <c r="L11">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="M11">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -2664,7 +2664,7 @@
         <v>72</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2983,7 +2983,7 @@
         <v>1212</v>
       </c>
       <c r="M10">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3024,7 +3024,7 @@
         <v>1774</v>
       </c>
       <c r="M11">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -3172,7 +3172,7 @@
         <v>504</v>
       </c>
       <c r="M3">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3254,7 +3254,7 @@
         <v>219</v>
       </c>
       <c r="M5">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3418,7 +3418,7 @@
         <v>344</v>
       </c>
       <c r="M9">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3500,7 +3500,7 @@
         <v>4436</v>
       </c>
       <c r="M11">
-        <v>517</v>
+        <v>521</v>
       </c>
     </row>
   </sheetData>
@@ -3712,7 +3712,7 @@
         <v>15</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3899,7 +3899,7 @@
         <v>180</v>
       </c>
       <c r="M10">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4369,7 +4369,7 @@
         <v>447</v>
       </c>
       <c r="M10">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4410,7 +4410,7 @@
         <v>739</v>
       </c>
       <c r="M11">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -4736,7 +4736,7 @@
         <v>119</v>
       </c>
       <c r="M8">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4859,7 +4859,7 @@
         <v>345</v>
       </c>
       <c r="M11">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -5007,7 +5007,7 @@
         <v>189</v>
       </c>
       <c r="M3">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5291,7 +5291,7 @@
         <v>495</v>
       </c>
       <c r="M10">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5332,7 +5332,7 @@
         <v>1490</v>
       </c>
       <c r="M11">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -5562,7 +5562,7 @@
         <v>125</v>
       </c>
       <c r="M5">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -5685,7 +5685,7 @@
         <v>461</v>
       </c>
       <c r="M8">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5767,7 +5767,7 @@
         <v>875</v>
       </c>
       <c r="M10">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5808,7 +5808,7 @@
         <v>2444</v>
       </c>
       <c r="M11">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -6158,7 +6158,7 @@
         <v>469</v>
       </c>
       <c r="M8">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6240,7 +6240,7 @@
         <v>864</v>
       </c>
       <c r="M10">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6281,7 +6281,7 @@
         <v>2096</v>
       </c>
       <c r="M11">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -6388,7 +6388,7 @@
         <v>929</v>
       </c>
       <c r="M2">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6470,7 +6470,7 @@
         <v>604</v>
       </c>
       <c r="M4">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6511,7 +6511,7 @@
         <v>267</v>
       </c>
       <c r="M5">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -6552,7 +6552,7 @@
         <v>780</v>
       </c>
       <c r="M6">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -6590,10 +6590,10 @@
         <v>2525</v>
       </c>
       <c r="L7">
-        <v>2419</v>
+        <v>2420</v>
       </c>
       <c r="M7">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6634,7 +6634,7 @@
         <v>4436</v>
       </c>
       <c r="M8">
-        <v>517</v>
+        <v>521</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6675,7 +6675,7 @@
         <v>448</v>
       </c>
       <c r="M9">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6716,7 +6716,7 @@
         <v>1155</v>
       </c>
       <c r="M10">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6757,7 +6757,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6798,7 +6798,7 @@
         <v>415</v>
       </c>
       <c r="M12">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -6880,7 +6880,7 @@
         <v>730</v>
       </c>
       <c r="M14">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -6921,7 +6921,7 @@
         <v>811</v>
       </c>
       <c r="M15">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -6962,7 +6962,7 @@
         <v>751</v>
       </c>
       <c r="M16">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7003,7 +7003,7 @@
         <v>130</v>
       </c>
       <c r="M17">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -7044,7 +7044,7 @@
         <v>644</v>
       </c>
       <c r="M18">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -7085,7 +7085,7 @@
         <v>2348</v>
       </c>
       <c r="M19">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -7126,7 +7126,7 @@
         <v>1705</v>
       </c>
       <c r="M20">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -7167,7 +7167,7 @@
         <v>280</v>
       </c>
       <c r="M21">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -7208,7 +7208,7 @@
         <v>391</v>
       </c>
       <c r="M22">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -7249,7 +7249,7 @@
         <v>1351</v>
       </c>
       <c r="M23">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -7413,7 +7413,7 @@
         <v>1244</v>
       </c>
       <c r="M27">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -7492,10 +7492,10 @@
         <v>3878</v>
       </c>
       <c r="L29">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="M29">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7577,7 +7577,7 @@
         <v>1014</v>
       </c>
       <c r="M31">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -7659,7 +7659,7 @@
         <v>2444</v>
       </c>
       <c r="M33">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -7700,7 +7700,7 @@
         <v>706</v>
       </c>
       <c r="M34">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -7741,7 +7741,7 @@
         <v>324</v>
       </c>
       <c r="M35">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -7782,7 +7782,7 @@
         <v>1431</v>
       </c>
       <c r="M36">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7823,7 +7823,7 @@
         <v>2340</v>
       </c>
       <c r="M37">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -7905,7 +7905,7 @@
         <v>182</v>
       </c>
       <c r="M39">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -8025,10 +8025,10 @@
         <v>3266</v>
       </c>
       <c r="L42">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="M42">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -8069,7 +8069,7 @@
         <v>1468</v>
       </c>
       <c r="M43">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -8110,7 +8110,7 @@
         <v>972</v>
       </c>
       <c r="M44">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -8274,7 +8274,7 @@
         <v>2778</v>
       </c>
       <c r="M48">
-        <v>360</v>
+        <v>382</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -8315,7 +8315,7 @@
         <v>1782</v>
       </c>
       <c r="M49">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -8397,7 +8397,7 @@
         <v>1453</v>
       </c>
       <c r="M51">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -8435,10 +8435,10 @@
         <v>1848</v>
       </c>
       <c r="L52">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="M52">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -8479,7 +8479,7 @@
         <v>1774</v>
       </c>
       <c r="M53">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -8520,7 +8520,7 @@
         <v>3846</v>
       </c>
       <c r="M54">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -8561,7 +8561,7 @@
         <v>1081</v>
       </c>
       <c r="M55">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -8602,7 +8602,7 @@
         <v>621</v>
       </c>
       <c r="M56">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -8643,7 +8643,7 @@
         <v>470</v>
       </c>
       <c r="M57">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -8725,7 +8725,7 @@
         <v>299</v>
       </c>
       <c r="M59">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -8766,7 +8766,7 @@
         <v>739</v>
       </c>
       <c r="M60">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -8883,13 +8883,13 @@
         <v>1053</v>
       </c>
       <c r="K63">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="L63">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="M63">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -8930,7 +8930,7 @@
         <v>949</v>
       </c>
       <c r="M64">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -8971,7 +8971,7 @@
         <v>1388</v>
       </c>
       <c r="M65">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -9012,7 +9012,7 @@
         <v>602</v>
       </c>
       <c r="M66">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -9053,7 +9053,7 @@
         <v>1927</v>
       </c>
       <c r="M67">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -9176,7 +9176,7 @@
         <v>656</v>
       </c>
       <c r="M70">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -9217,7 +9217,7 @@
         <v>345</v>
       </c>
       <c r="M71">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="72" spans="1:13">
@@ -9258,7 +9258,7 @@
         <v>667</v>
       </c>
       <c r="M72">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="73" spans="1:13">
@@ -9299,7 +9299,7 @@
         <v>1356</v>
       </c>
       <c r="M73">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -9340,7 +9340,7 @@
         <v>314</v>
       </c>
       <c r="M74">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -9381,7 +9381,7 @@
         <v>428</v>
       </c>
       <c r="M75">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -9419,10 +9419,10 @@
         <v>3059</v>
       </c>
       <c r="L76">
-        <v>3358</v>
+        <v>3360</v>
       </c>
       <c r="M76">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -9501,10 +9501,10 @@
         <v>1940</v>
       </c>
       <c r="L78">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="M78">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -9545,7 +9545,7 @@
         <v>2096</v>
       </c>
       <c r="M79">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -9586,7 +9586,7 @@
         <v>477</v>
       </c>
       <c r="M80">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -9627,7 +9627,7 @@
         <v>186</v>
       </c>
       <c r="M81">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -9668,7 +9668,7 @@
         <v>233</v>
       </c>
       <c r="M82">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="83" spans="1:13">
@@ -9709,7 +9709,7 @@
         <v>1490</v>
       </c>
       <c r="M83">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -9791,7 +9791,7 @@
         <v>3420</v>
       </c>
       <c r="M85">
-        <v>413</v>
+        <v>420</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -9832,7 +9832,7 @@
         <v>905</v>
       </c>
       <c r="M86">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -9873,7 +9873,7 @@
         <v>440</v>
       </c>
       <c r="M87">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -9914,7 +9914,7 @@
         <v>880</v>
       </c>
       <c r="M88">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -9955,7 +9955,7 @@
         <v>2047</v>
       </c>
       <c r="M89">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -9996,7 +9996,7 @@
         <v>1095</v>
       </c>
       <c r="M90">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -10078,7 +10078,7 @@
         <v>318</v>
       </c>
       <c r="M92">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="93" spans="1:13">
@@ -10119,7 +10119,7 @@
         <v>810</v>
       </c>
       <c r="M93">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="94" spans="1:13">
@@ -10160,7 +10160,7 @@
         <v>2677</v>
       </c>
       <c r="M94">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -10201,7 +10201,7 @@
         <v>1239</v>
       </c>
       <c r="M95">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -10242,7 +10242,7 @@
         <v>1361</v>
       </c>
       <c r="M96">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -10283,7 +10283,7 @@
         <v>1730</v>
       </c>
       <c r="M97">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -10324,7 +10324,7 @@
         <v>1134</v>
       </c>
       <c r="M98">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="99" spans="1:13">
@@ -10365,7 +10365,7 @@
         <v>1514</v>
       </c>
       <c r="M99">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -10441,13 +10441,13 @@
         <v>124135</v>
       </c>
       <c r="K101">
-        <v>118747</v>
+        <v>118749</v>
       </c>
       <c r="L101">
-        <v>104077</v>
+        <v>104081</v>
       </c>
       <c r="M101">
-        <v>12846</v>
+        <v>13086</v>
       </c>
     </row>
   </sheetData>
@@ -10954,7 +10954,7 @@
         <v>266</v>
       </c>
       <c r="M10">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -10995,7 +10995,7 @@
         <v>428</v>
       </c>
       <c r="M11">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -11690,6 +11690,9 @@
       <c r="L6">
         <v>15</v>
       </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
@@ -11764,7 +11767,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11846,7 +11849,7 @@
         <v>546</v>
       </c>
       <c r="M10">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -11887,7 +11890,7 @@
         <v>949</v>
       </c>
       <c r="M11">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -11994,7 +11997,7 @@
         <v>107</v>
       </c>
       <c r="M2">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -12035,7 +12038,7 @@
         <v>101</v>
       </c>
       <c r="M3">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -12117,7 +12120,7 @@
         <v>147</v>
       </c>
       <c r="M5">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -12240,7 +12243,7 @@
         <v>285</v>
       </c>
       <c r="M8">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -12363,7 +12366,7 @@
         <v>1239</v>
       </c>
       <c r="M11">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -12795,7 +12798,7 @@
         <v>900</v>
       </c>
       <c r="M10">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12836,7 +12839,7 @@
         <v>2340</v>
       </c>
       <c r="M11">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -12984,7 +12987,7 @@
         <v>136</v>
       </c>
       <c r="M3">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -13066,7 +13069,7 @@
         <v>102</v>
       </c>
       <c r="M5">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13186,7 +13189,7 @@
         <v>233</v>
       </c>
       <c r="M8">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13227,7 +13230,7 @@
         <v>105</v>
       </c>
       <c r="M9">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -13268,7 +13271,7 @@
         <v>605</v>
       </c>
       <c r="M10">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13309,7 +13312,7 @@
         <v>1388</v>
       </c>
       <c r="M11">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -13726,7 +13729,7 @@
         <v>818</v>
       </c>
       <c r="M10">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13767,7 +13770,7 @@
         <v>1244</v>
       </c>
       <c r="M11">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -14120,7 +14123,7 @@
         <v>288</v>
       </c>
       <c r="M8">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -14161,7 +14164,7 @@
         <v>80</v>
       </c>
       <c r="M9">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -14202,7 +14205,7 @@
         <v>753</v>
       </c>
       <c r="M10">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -14243,7 +14246,7 @@
         <v>1514</v>
       </c>
       <c r="M11">
-        <v>211</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -15133,7 +15136,7 @@
         <v>606</v>
       </c>
       <c r="M10">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15174,7 +15177,7 @@
         <v>1014</v>
       </c>
       <c r="M11">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -15512,7 +15515,7 @@
         <v>121</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -15591,7 +15594,7 @@
         <v>428</v>
       </c>
       <c r="M10">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15632,7 +15635,7 @@
         <v>730</v>
       </c>
       <c r="M11">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -15780,7 +15783,7 @@
         <v>295</v>
       </c>
       <c r="M3">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -15985,7 +15988,7 @@
         <v>322</v>
       </c>
       <c r="M8">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16067,7 +16070,7 @@
         <v>739</v>
       </c>
       <c r="M10">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16108,7 +16111,7 @@
         <v>1927</v>
       </c>
       <c r="M11">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -16910,7 +16913,7 @@
         <v>358</v>
       </c>
       <c r="M8">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16992,7 +16995,7 @@
         <v>1963</v>
       </c>
       <c r="M10">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17033,7 +17036,7 @@
         <v>2677</v>
       </c>
       <c r="M11">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -17456,10 +17459,10 @@
         <v>2251</v>
       </c>
       <c r="L10">
-        <v>2712</v>
+        <v>2714</v>
       </c>
       <c r="M10">
-        <v>309</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17497,10 +17500,10 @@
         <v>3059</v>
       </c>
       <c r="L11">
-        <v>3358</v>
+        <v>3360</v>
       </c>
       <c r="M11">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>
@@ -17902,7 +17905,7 @@
         <v>304</v>
       </c>
       <c r="M10">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17943,7 +17946,7 @@
         <v>440</v>
       </c>
       <c r="M11">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -19204,7 +19207,7 @@
         <v>592</v>
       </c>
       <c r="M10">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19245,7 +19248,7 @@
         <v>751</v>
       </c>
       <c r="M11">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -19574,7 +19577,7 @@
         <v>165</v>
       </c>
       <c r="M8">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -19656,7 +19659,7 @@
         <v>1379</v>
       </c>
       <c r="M10">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19697,7 +19700,7 @@
         <v>1782</v>
       </c>
       <c r="M11">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -19804,7 +19807,7 @@
         <v>45</v>
       </c>
       <c r="M2">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20126,7 +20129,7 @@
         <v>1116</v>
       </c>
       <c r="M10">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20167,7 +20170,7 @@
         <v>1730</v>
       </c>
       <c r="M11">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -20517,7 +20520,7 @@
         <v>252</v>
       </c>
       <c r="M8">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20599,7 +20602,7 @@
         <v>763</v>
       </c>
       <c r="M10">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20640,7 +20643,7 @@
         <v>1361</v>
       </c>
       <c r="M11">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -20990,7 +20993,7 @@
         <v>183</v>
       </c>
       <c r="M8">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21072,7 +21075,7 @@
         <v>586</v>
       </c>
       <c r="M10">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21113,7 +21116,7 @@
         <v>1081</v>
       </c>
       <c r="M11">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -21463,7 +21466,7 @@
         <v>361</v>
       </c>
       <c r="M8">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21545,7 +21548,7 @@
         <v>2938</v>
       </c>
       <c r="M10">
-        <v>345</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21586,7 +21589,7 @@
         <v>3846</v>
       </c>
       <c r="M11">
-        <v>471</v>
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -22015,7 +22018,7 @@
         <v>904</v>
       </c>
       <c r="M10">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22056,7 +22059,7 @@
         <v>1356</v>
       </c>
       <c r="M11">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -22163,7 +22166,7 @@
         <v>371</v>
       </c>
       <c r="M2">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -22324,7 +22327,7 @@
         <v>74</v>
       </c>
       <c r="L6">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M6">
         <v>10</v>
@@ -22409,7 +22412,7 @@
         <v>644</v>
       </c>
       <c r="M8">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22491,7 +22494,7 @@
         <v>1276</v>
       </c>
       <c r="M10">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22529,10 +22532,10 @@
         <v>3878</v>
       </c>
       <c r="L11">
-        <v>3376</v>
+        <v>3377</v>
       </c>
       <c r="M11">
-        <v>424</v>
+        <v>430</v>
       </c>
     </row>
   </sheetData>
@@ -22639,7 +22642,7 @@
         <v>42</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -22756,7 +22759,7 @@
         <v>207</v>
       </c>
       <c r="M5">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -22867,7 +22870,7 @@
         <v>253</v>
       </c>
       <c r="M8">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22949,7 +22952,7 @@
         <v>2038</v>
       </c>
       <c r="M10">
-        <v>272</v>
+        <v>289</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22990,7 +22993,7 @@
         <v>2778</v>
       </c>
       <c r="M11">
-        <v>360</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -23097,7 +23100,7 @@
         <v>214</v>
       </c>
       <c r="M2">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -23343,7 +23346,7 @@
         <v>412</v>
       </c>
       <c r="M8">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23425,7 +23428,7 @@
         <v>1136</v>
       </c>
       <c r="M10">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23466,7 +23469,7 @@
         <v>2348</v>
       </c>
       <c r="M11">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -23684,7 +23687,7 @@
         <v>71</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -23862,7 +23865,7 @@
         <v>383</v>
       </c>
       <c r="M10">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23903,7 +23906,7 @@
         <v>602</v>
       </c>
       <c r="M11">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -24326,7 +24329,7 @@
         <v>604</v>
       </c>
       <c r="M10">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24367,7 +24370,7 @@
         <v>972</v>
       </c>
       <c r="M11">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -24717,10 +24720,10 @@
         <v>719</v>
       </c>
       <c r="L8">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="M8">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24802,7 +24805,7 @@
         <v>1167</v>
       </c>
       <c r="M10">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24840,10 +24843,10 @@
         <v>3266</v>
       </c>
       <c r="L11">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="M11">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -25169,7 +25172,7 @@
         <v>92</v>
       </c>
       <c r="M8">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -25248,7 +25251,7 @@
         <v>193</v>
       </c>
       <c r="M10">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25289,7 +25292,7 @@
         <v>391</v>
       </c>
       <c r="M11">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -25396,7 +25399,7 @@
         <v>245</v>
       </c>
       <c r="M2">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -25560,7 +25563,7 @@
         <v>46</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -25639,7 +25642,7 @@
         <v>588</v>
       </c>
       <c r="L8">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="M8">
         <v>72</v>
@@ -25724,7 +25727,7 @@
         <v>941</v>
       </c>
       <c r="M10">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25762,10 +25765,10 @@
         <v>2525</v>
       </c>
       <c r="L11">
-        <v>2419</v>
+        <v>2420</v>
       </c>
       <c r="M11">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -26191,7 +26194,7 @@
         <v>320</v>
       </c>
       <c r="M10">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26232,7 +26235,7 @@
         <v>780</v>
       </c>
       <c r="M11">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -26920,7 +26923,7 @@
         <v>78</v>
       </c>
       <c r="M5">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -27122,7 +27125,7 @@
         <v>641</v>
       </c>
       <c r="M10">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -27163,7 +27166,7 @@
         <v>1431</v>
       </c>
       <c r="M11">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -27993,7 +27996,7 @@
         <v>826</v>
       </c>
       <c r="M10">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28034,7 +28037,7 @@
         <v>1155</v>
       </c>
       <c r="M11">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -28284,7 +28287,7 @@
         <v>72</v>
       </c>
       <c r="M6">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -28427,7 +28430,7 @@
         <v>661</v>
       </c>
       <c r="M10">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28468,7 +28471,7 @@
         <v>905</v>
       </c>
       <c r="M11">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -28616,7 +28619,7 @@
         <v>92</v>
       </c>
       <c r="M3">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -28733,7 +28736,7 @@
         <v>33</v>
       </c>
       <c r="L6">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M6">
         <v>9</v>
@@ -28897,7 +28900,7 @@
         <v>979</v>
       </c>
       <c r="M10">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28935,10 +28938,10 @@
         <v>1940</v>
       </c>
       <c r="L11">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="M11">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -29940,7 +29943,7 @@
         <v>70</v>
       </c>
       <c r="M2">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -30227,7 +30230,7 @@
         <v>38</v>
       </c>
       <c r="M9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -30309,7 +30312,7 @@
         <v>811</v>
       </c>
       <c r="M11">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -30738,7 +30741,7 @@
         <v>1042</v>
       </c>
       <c r="M10">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30779,7 +30782,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -31202,7 +31205,7 @@
         <v>722</v>
       </c>
       <c r="M10">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31243,7 +31246,7 @@
         <v>1351</v>
       </c>
       <c r="M11">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -31826,7 +31829,7 @@
         <v>83</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -32066,7 +32069,7 @@
         <v>311</v>
       </c>
       <c r="M8">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -32189,7 +32192,7 @@
         <v>1453</v>
       </c>
       <c r="M11">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -32624,7 +32627,7 @@
         <v>735</v>
       </c>
       <c r="M10">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32665,7 +32668,7 @@
         <v>1705</v>
       </c>
       <c r="M11">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -33046,7 +33049,7 @@
         <v>169</v>
       </c>
       <c r="M10">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33087,7 +33090,7 @@
         <v>280</v>
       </c>
       <c r="M11">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -33652,7 +33655,7 @@
         <v>79</v>
       </c>
       <c r="M2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -33853,6 +33856,9 @@
       <c r="L7">
         <v>3</v>
       </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
@@ -33974,7 +33980,7 @@
         <v>483</v>
       </c>
       <c r="M10">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34015,7 +34021,7 @@
         <v>1095</v>
       </c>
       <c r="M11">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -34700,7 +34706,7 @@
         <v>52</v>
       </c>
       <c r="M5">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -34808,7 +34814,7 @@
         <v>156</v>
       </c>
       <c r="M8">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -34890,7 +34896,7 @@
         <v>490</v>
       </c>
       <c r="M10">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34931,7 +34937,7 @@
         <v>810</v>
       </c>
       <c r="M11">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -35038,7 +35044,7 @@
         <v>51</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -35079,7 +35085,7 @@
         <v>51</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -35357,7 +35363,7 @@
         <v>267</v>
       </c>
       <c r="M10">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35398,7 +35404,7 @@
         <v>644</v>
       </c>
       <c r="M11">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -35782,7 +35788,7 @@
         <v>530</v>
       </c>
       <c r="M10">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35823,7 +35829,7 @@
         <v>656</v>
       </c>
       <c r="M11">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -36659,7 +36665,7 @@
         <v>585</v>
       </c>
       <c r="M10">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36700,7 +36706,7 @@
         <v>621</v>
       </c>
       <c r="M11">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -37102,7 +37108,7 @@
         <v>121</v>
       </c>
       <c r="M10">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -37143,7 +37149,7 @@
         <v>267</v>
       </c>
       <c r="M11">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -37490,7 +37496,7 @@
         <v>156</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -37613,7 +37619,7 @@
         <v>929</v>
       </c>
       <c r="M11">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -37831,7 +37837,7 @@
         <v>53</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -38021,7 +38027,7 @@
         <v>454</v>
       </c>
       <c r="M10">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38062,7 +38068,7 @@
         <v>667</v>
       </c>
       <c r="M11">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -38461,7 +38467,7 @@
         <v>1039</v>
       </c>
       <c r="M10">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38502,7 +38508,7 @@
         <v>1468</v>
       </c>
       <c r="M11">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -38713,6 +38719,9 @@
       <c r="L5">
         <v>8</v>
       </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
@@ -38936,7 +38945,7 @@
         <v>130</v>
       </c>
       <c r="M11">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -39344,7 +39353,7 @@
         <v>413</v>
       </c>
       <c r="M10">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -39385,7 +39394,7 @@
         <v>604</v>
       </c>
       <c r="M11">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -39588,7 +39597,7 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -39807,7 +39816,7 @@
         <v>477</v>
       </c>
       <c r="M11">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -40151,7 +40160,7 @@
         <v>142</v>
       </c>
       <c r="M8">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -40274,7 +40283,7 @@
         <v>706</v>
       </c>
       <c r="M11">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -40422,7 +40431,7 @@
         <v>85</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -40545,7 +40554,7 @@
         <v>46</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -40703,7 +40712,7 @@
         <v>1436</v>
       </c>
       <c r="M10">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40744,7 +40753,7 @@
         <v>2047</v>
       </c>
       <c r="M11">
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -41107,7 +41116,7 @@
         <v>267</v>
       </c>
       <c r="M10">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -41148,7 +41157,7 @@
         <v>324</v>
       </c>
       <c r="M11">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -42558,7 +42567,7 @@
         <v>65</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -42751,7 +42760,7 @@
         <v>795</v>
       </c>
       <c r="M10">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -42792,7 +42801,7 @@
         <v>1134</v>
       </c>
       <c r="M11">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -43303,7 +43312,7 @@
         <v>29</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -43660,7 +43669,7 @@
         <v>318</v>
       </c>
       <c r="M11">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -44442,7 +44451,7 @@
         <v>152</v>
       </c>
       <c r="M10">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -44483,7 +44492,7 @@
         <v>233</v>
       </c>
       <c r="M11">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -44833,7 +44842,7 @@
         <v>105</v>
       </c>
       <c r="M8">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -44956,7 +44965,7 @@
         <v>448</v>
       </c>
       <c r="M11">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -45104,7 +45113,7 @@
         <v>448</v>
       </c>
       <c r="M3">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -45309,7 +45318,7 @@
         <v>642</v>
       </c>
       <c r="M8">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45350,7 +45359,7 @@
         <v>228</v>
       </c>
       <c r="M9">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -45391,7 +45400,7 @@
         <v>1371</v>
       </c>
       <c r="M10">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45432,7 +45441,7 @@
         <v>3420</v>
       </c>
       <c r="M11">
-        <v>413</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>
@@ -45746,7 +45755,7 @@
         <v>65</v>
       </c>
       <c r="M8">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45869,7 +45878,7 @@
         <v>299</v>
       </c>
       <c r="M11">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -46171,6 +46180,9 @@
       <c r="L7">
         <v>4</v>
       </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
@@ -46210,7 +46222,7 @@
         <v>146</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -46251,7 +46263,7 @@
         <v>182</v>
       </c>
       <c r="M9">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -46665,7 +46677,7 @@
         <v>296</v>
       </c>
       <c r="M10">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -46706,7 +46718,7 @@
         <v>470</v>
       </c>
       <c r="M11">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -46813,7 +46825,7 @@
         <v>67</v>
       </c>
       <c r="M2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -47132,7 +47144,7 @@
         <v>435</v>
       </c>
       <c r="M10">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -47173,7 +47185,7 @@
         <v>880</v>
       </c>
       <c r="M11">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -47539,7 +47551,7 @@
         <v>268</v>
       </c>
       <c r="M10">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -47580,7 +47592,7 @@
         <v>314</v>
       </c>
       <c r="M11">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -48247,7 +48259,7 @@
         <v>28</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -48367,7 +48379,7 @@
         <v>186</v>
       </c>
       <c r="M11">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -49141,7 +49153,7 @@
         <v>253</v>
       </c>
       <c r="M10">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -49182,7 +49194,7 @@
         <v>415</v>
       </c>
       <c r="M11">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-03-31
</commit_message>
<xml_diff>
--- a/output/index-crime-full-year.xlsx
+++ b/output/index-crime-full-year.xlsx
@@ -913,7 +913,7 @@
         <v>6580</v>
       </c>
       <c r="M2">
-        <v>1314</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -951,10 +951,10 @@
         <v>8178</v>
       </c>
       <c r="L3">
-        <v>7115</v>
+        <v>7116</v>
       </c>
       <c r="M3">
-        <v>1440</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -995,7 +995,7 @@
         <v>373</v>
       </c>
       <c r="M4">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1036,7 +1036,7 @@
         <v>6198</v>
       </c>
       <c r="M5">
-        <v>1114</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1050,10 +1050,10 @@
         <v>1880</v>
       </c>
       <c r="D6">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="E6">
-        <v>2072</v>
+        <v>2071</v>
       </c>
       <c r="F6">
         <v>1935</v>
@@ -1071,13 +1071,13 @@
         <v>1894</v>
       </c>
       <c r="K6">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="L6">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="M6">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1118,7 +1118,7 @@
         <v>426</v>
       </c>
       <c r="M7">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1159,7 +1159,7 @@
         <v>17237</v>
       </c>
       <c r="M8">
-        <v>4054</v>
+        <v>4099</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1200,7 +1200,7 @@
         <v>5809</v>
       </c>
       <c r="M9">
-        <v>1019</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1235,13 +1235,13 @@
         <v>57511</v>
       </c>
       <c r="K10">
-        <v>61312</v>
+        <v>61313</v>
       </c>
       <c r="L10">
-        <v>58623</v>
+        <v>58624</v>
       </c>
       <c r="M10">
-        <v>12445</v>
+        <v>12628</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1255,10 +1255,10 @@
         <v>116142</v>
       </c>
       <c r="D11">
-        <v>117407</v>
+        <v>117408</v>
       </c>
       <c r="E11">
-        <v>113474</v>
+        <v>113473</v>
       </c>
       <c r="F11">
         <v>105620</v>
@@ -1276,13 +1276,13 @@
         <v>124139</v>
       </c>
       <c r="K11">
-        <v>118754</v>
+        <v>118756</v>
       </c>
       <c r="L11">
-        <v>104163</v>
+        <v>104164</v>
       </c>
       <c r="M11">
-        <v>21956</v>
+        <v>22254</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1389,7 @@
         <v>145</v>
       </c>
       <c r="M2">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1430,7 +1430,7 @@
         <v>142</v>
       </c>
       <c r="M3">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1676,7 +1676,7 @@
         <v>128</v>
       </c>
       <c r="M9">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1717,7 +1717,7 @@
         <v>683</v>
       </c>
       <c r="M10">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1758,7 +1758,7 @@
         <v>1410</v>
       </c>
       <c r="M11">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -2519,7 +2519,7 @@
         <v>339</v>
       </c>
       <c r="M10">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2560,7 +2560,7 @@
         <v>473</v>
       </c>
       <c r="M11">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2667,7 +2667,7 @@
         <v>72</v>
       </c>
       <c r="M2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2986,7 +2986,7 @@
         <v>1203</v>
       </c>
       <c r="M10">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3027,7 +3027,7 @@
         <v>1754</v>
       </c>
       <c r="M11">
-        <v>368</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -3175,7 +3175,7 @@
         <v>504</v>
       </c>
       <c r="M3">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -3257,7 +3257,7 @@
         <v>217</v>
       </c>
       <c r="M5">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3298,7 +3298,7 @@
         <v>104</v>
       </c>
       <c r="M6">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3380,7 +3380,7 @@
         <v>777</v>
       </c>
       <c r="M8">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3462,7 +3462,7 @@
         <v>1966</v>
       </c>
       <c r="M10">
-        <v>363</v>
+        <v>377</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3503,7 +3503,7 @@
         <v>4421</v>
       </c>
       <c r="M11">
-        <v>879</v>
+        <v>897</v>
       </c>
     </row>
   </sheetData>
@@ -3820,7 +3820,7 @@
         <v>55</v>
       </c>
       <c r="M8">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3943,7 +3943,7 @@
         <v>300</v>
       </c>
       <c r="M11">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -4208,7 +4208,7 @@
         <v>13</v>
       </c>
       <c r="L6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M6">
         <v>2</v>
@@ -4375,7 +4375,7 @@
         <v>447</v>
       </c>
       <c r="M10">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4413,10 +4413,10 @@
         <v>786</v>
       </c>
       <c r="L11">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="M11">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -4827,7 +4827,7 @@
         <v>161</v>
       </c>
       <c r="M10">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4868,7 +4868,7 @@
         <v>346</v>
       </c>
       <c r="M11">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -4975,7 +4975,7 @@
         <v>151</v>
       </c>
       <c r="M2">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -5098,7 +5098,7 @@
         <v>125</v>
       </c>
       <c r="M5">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -5218,7 +5218,7 @@
         <v>377</v>
       </c>
       <c r="M8">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5300,7 +5300,7 @@
         <v>492</v>
       </c>
       <c r="M10">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5341,7 +5341,7 @@
         <v>1485</v>
       </c>
       <c r="M11">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>
@@ -5448,7 +5448,7 @@
         <v>266</v>
       </c>
       <c r="M2">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -5489,7 +5489,7 @@
         <v>342</v>
       </c>
       <c r="M3">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5653,7 +5653,7 @@
         <v>25</v>
       </c>
       <c r="M7">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -5776,7 +5776,7 @@
         <v>874</v>
       </c>
       <c r="M10">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5817,7 +5817,7 @@
         <v>2442</v>
       </c>
       <c r="M11">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -5924,7 +5924,7 @@
         <v>187</v>
       </c>
       <c r="M2">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6047,7 +6047,7 @@
         <v>149</v>
       </c>
       <c r="M5">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -6252,7 +6252,7 @@
         <v>861</v>
       </c>
       <c r="M10">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6293,7 +6293,7 @@
         <v>2091</v>
       </c>
       <c r="M11">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
   </sheetData>
@@ -6400,7 +6400,7 @@
         <v>924</v>
       </c>
       <c r="M2">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6482,7 +6482,7 @@
         <v>597</v>
       </c>
       <c r="M4">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6564,7 +6564,7 @@
         <v>778</v>
       </c>
       <c r="M6">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -6605,7 +6605,7 @@
         <v>2409</v>
       </c>
       <c r="M7">
-        <v>441</v>
+        <v>446</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6646,7 +6646,7 @@
         <v>4421</v>
       </c>
       <c r="M8">
-        <v>879</v>
+        <v>897</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6687,7 +6687,7 @@
         <v>442</v>
       </c>
       <c r="M9">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6728,7 +6728,7 @@
         <v>1154</v>
       </c>
       <c r="M10">
-        <v>294</v>
+        <v>298</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6769,7 +6769,7 @@
         <v>1776</v>
       </c>
       <c r="M11">
-        <v>439</v>
+        <v>443</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6851,7 +6851,7 @@
         <v>266</v>
       </c>
       <c r="M13">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -6933,7 +6933,7 @@
         <v>811</v>
       </c>
       <c r="M15">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -6974,7 +6974,7 @@
         <v>745</v>
       </c>
       <c r="M16">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7097,7 +7097,7 @@
         <v>2329</v>
       </c>
       <c r="M19">
-        <v>473</v>
+        <v>481</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -7138,7 +7138,7 @@
         <v>1695</v>
       </c>
       <c r="M20">
-        <v>368</v>
+        <v>374</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -7220,7 +7220,7 @@
         <v>386</v>
       </c>
       <c r="M22">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -7261,7 +7261,7 @@
         <v>1351</v>
       </c>
       <c r="M23">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -7343,7 +7343,7 @@
         <v>580</v>
       </c>
       <c r="M25">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -7384,7 +7384,7 @@
         <v>237</v>
       </c>
       <c r="M26">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -7507,7 +7507,7 @@
         <v>3361</v>
       </c>
       <c r="M29">
-        <v>673</v>
+        <v>681</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7548,7 +7548,7 @@
         <v>276</v>
       </c>
       <c r="M30">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -7589,7 +7589,7 @@
         <v>1013</v>
       </c>
       <c r="M31">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -7630,7 +7630,7 @@
         <v>180</v>
       </c>
       <c r="M32">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -7671,7 +7671,7 @@
         <v>2442</v>
       </c>
       <c r="M33">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -7712,7 +7712,7 @@
         <v>702</v>
       </c>
       <c r="M34">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -7753,7 +7753,7 @@
         <v>322</v>
       </c>
       <c r="M35">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -7794,7 +7794,7 @@
         <v>1424</v>
       </c>
       <c r="M36">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7835,7 +7835,7 @@
         <v>2334</v>
       </c>
       <c r="M37">
-        <v>466</v>
+        <v>472</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -7876,7 +7876,7 @@
         <v>134</v>
       </c>
       <c r="M38">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -7958,7 +7958,7 @@
         <v>329</v>
       </c>
       <c r="M40">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -7999,7 +7999,7 @@
         <v>361</v>
       </c>
       <c r="M41">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -8040,7 +8040,7 @@
         <v>2488</v>
       </c>
       <c r="M42">
-        <v>559</v>
+        <v>567</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -8081,7 +8081,7 @@
         <v>1460</v>
       </c>
       <c r="M43">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -8122,7 +8122,7 @@
         <v>968</v>
       </c>
       <c r="M44">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -8204,7 +8204,7 @@
         <v>300</v>
       </c>
       <c r="M46">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -8245,7 +8245,7 @@
         <v>939</v>
       </c>
       <c r="M47">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -8286,7 +8286,7 @@
         <v>2765</v>
       </c>
       <c r="M48">
-        <v>658</v>
+        <v>664</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -8327,7 +8327,7 @@
         <v>1779</v>
       </c>
       <c r="M49">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -8368,7 +8368,7 @@
         <v>1015</v>
       </c>
       <c r="M50">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -8409,7 +8409,7 @@
         <v>1445</v>
       </c>
       <c r="M51">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -8450,7 +8450,7 @@
         <v>1410</v>
       </c>
       <c r="M52">
-        <v>281</v>
+        <v>285</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -8491,7 +8491,7 @@
         <v>1754</v>
       </c>
       <c r="M53">
-        <v>368</v>
+        <v>377</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -8532,7 +8532,7 @@
         <v>3829</v>
       </c>
       <c r="M54">
-        <v>810</v>
+        <v>828</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -8573,7 +8573,7 @@
         <v>1078</v>
       </c>
       <c r="M55">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -8614,7 +8614,7 @@
         <v>620</v>
       </c>
       <c r="M56">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -8655,7 +8655,7 @@
         <v>467</v>
       </c>
       <c r="M57">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -8696,7 +8696,7 @@
         <v>143</v>
       </c>
       <c r="M58">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -8737,7 +8737,7 @@
         <v>298</v>
       </c>
       <c r="M59">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -8775,10 +8775,10 @@
         <v>786</v>
       </c>
       <c r="L60">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="M60">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -8874,10 +8874,10 @@
         <v>1234</v>
       </c>
       <c r="D63">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="E63">
-        <v>2124</v>
+        <v>2123</v>
       </c>
       <c r="F63">
         <v>1385</v>
@@ -8895,13 +8895,13 @@
         <v>1057</v>
       </c>
       <c r="K63">
-        <v>877</v>
+        <v>879</v>
       </c>
       <c r="L63">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="M63">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -8942,7 +8942,7 @@
         <v>947</v>
       </c>
       <c r="M64">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -8983,7 +8983,7 @@
         <v>1383</v>
       </c>
       <c r="M65">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -9024,7 +9024,7 @@
         <v>601</v>
       </c>
       <c r="M66">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -9065,7 +9065,7 @@
         <v>1919</v>
       </c>
       <c r="M67">
-        <v>424</v>
+        <v>428</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -9106,7 +9106,7 @@
         <v>500</v>
       </c>
       <c r="M68">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -9147,7 +9147,7 @@
         <v>473</v>
       </c>
       <c r="M69">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -9188,7 +9188,7 @@
         <v>654</v>
       </c>
       <c r="M70">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -9229,7 +9229,7 @@
         <v>346</v>
       </c>
       <c r="M71">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="72" spans="1:13">
@@ -9270,7 +9270,7 @@
         <v>662</v>
       </c>
       <c r="M72">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="73" spans="1:13">
@@ -9311,7 +9311,7 @@
         <v>1350</v>
       </c>
       <c r="M73">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -9393,7 +9393,7 @@
         <v>427</v>
       </c>
       <c r="M75">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -9434,7 +9434,7 @@
         <v>3351</v>
       </c>
       <c r="M76">
-        <v>666</v>
+        <v>677</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -9475,7 +9475,7 @@
         <v>373</v>
       </c>
       <c r="M77">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -9513,10 +9513,10 @@
         <v>1939</v>
       </c>
       <c r="L78">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="M78">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -9557,7 +9557,7 @@
         <v>2091</v>
       </c>
       <c r="M79">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -9598,7 +9598,7 @@
         <v>470</v>
       </c>
       <c r="M80">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -9680,7 +9680,7 @@
         <v>231</v>
       </c>
       <c r="M82">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="83" spans="1:13">
@@ -9721,7 +9721,7 @@
         <v>1485</v>
       </c>
       <c r="M83">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -9803,7 +9803,7 @@
         <v>3397</v>
       </c>
       <c r="M85">
-        <v>715</v>
+        <v>729</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -9844,7 +9844,7 @@
         <v>902</v>
       </c>
       <c r="M86">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -9885,7 +9885,7 @@
         <v>437</v>
       </c>
       <c r="M87">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -9926,7 +9926,7 @@
         <v>874</v>
       </c>
       <c r="M88">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -9967,7 +9967,7 @@
         <v>2036</v>
       </c>
       <c r="M89">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -10008,7 +10008,7 @@
         <v>1090</v>
       </c>
       <c r="M90">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -10049,7 +10049,7 @@
         <v>966</v>
       </c>
       <c r="M91">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -10131,7 +10131,7 @@
         <v>803</v>
       </c>
       <c r="M93">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="94" spans="1:13">
@@ -10172,7 +10172,7 @@
         <v>2666</v>
       </c>
       <c r="M94">
-        <v>602</v>
+        <v>608</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -10213,7 +10213,7 @@
         <v>1237</v>
       </c>
       <c r="M95">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -10254,7 +10254,7 @@
         <v>1358</v>
       </c>
       <c r="M96">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -10295,7 +10295,7 @@
         <v>1719</v>
       </c>
       <c r="M97">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -10336,7 +10336,7 @@
         <v>1128</v>
       </c>
       <c r="M98">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="99" spans="1:13">
@@ -10377,7 +10377,7 @@
         <v>1505</v>
       </c>
       <c r="M99">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -10418,7 +10418,7 @@
         <v>277</v>
       </c>
       <c r="M100">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="101" spans="1:13">
@@ -10432,10 +10432,10 @@
         <v>116142</v>
       </c>
       <c r="D101">
-        <v>117407</v>
+        <v>117408</v>
       </c>
       <c r="E101">
-        <v>113474</v>
+        <v>113473</v>
       </c>
       <c r="F101">
         <v>105620</v>
@@ -10453,13 +10453,13 @@
         <v>124139</v>
       </c>
       <c r="K101">
-        <v>118754</v>
+        <v>118756</v>
       </c>
       <c r="L101">
-        <v>104163</v>
+        <v>104164</v>
       </c>
       <c r="M101">
-        <v>21956</v>
+        <v>22254</v>
       </c>
     </row>
   </sheetData>
@@ -10966,7 +10966,7 @@
         <v>265</v>
       </c>
       <c r="M10">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -11007,7 +11007,7 @@
         <v>427</v>
       </c>
       <c r="M11">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -11321,7 +11321,7 @@
         <v>103</v>
       </c>
       <c r="M8">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11444,7 +11444,7 @@
         <v>329</v>
       </c>
       <c r="M11">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -11779,7 +11779,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11902,7 +11902,7 @@
         <v>947</v>
       </c>
       <c r="M11">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -12009,7 +12009,7 @@
         <v>105</v>
       </c>
       <c r="M2">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -12132,7 +12132,7 @@
         <v>147</v>
       </c>
       <c r="M5">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -12214,7 +12214,7 @@
         <v>7</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -12255,7 +12255,7 @@
         <v>285</v>
       </c>
       <c r="M8">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -12378,7 +12378,7 @@
         <v>1237</v>
       </c>
       <c r="M11">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -12485,7 +12485,7 @@
         <v>250</v>
       </c>
       <c r="M2">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -12526,7 +12526,7 @@
         <v>294</v>
       </c>
       <c r="M3">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -12813,7 +12813,7 @@
         <v>901</v>
       </c>
       <c r="M10">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12854,7 +12854,7 @@
         <v>2334</v>
       </c>
       <c r="M11">
-        <v>466</v>
+        <v>472</v>
       </c>
     </row>
   </sheetData>
@@ -13002,7 +13002,7 @@
         <v>137</v>
       </c>
       <c r="M3">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -13289,7 +13289,7 @@
         <v>601</v>
       </c>
       <c r="M10">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13330,7 +13330,7 @@
         <v>1383</v>
       </c>
       <c r="M11">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>
@@ -13936,7 +13936,7 @@
         <v>150</v>
       </c>
       <c r="M3">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -14018,7 +14018,7 @@
         <v>91</v>
       </c>
       <c r="M5">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -14141,7 +14141,7 @@
         <v>286</v>
       </c>
       <c r="M8">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -14223,7 +14223,7 @@
         <v>749</v>
       </c>
       <c r="M10">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -14264,7 +14264,7 @@
         <v>1505</v>
       </c>
       <c r="M11">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -14599,7 +14599,7 @@
         <v>59</v>
       </c>
       <c r="M8">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -14722,7 +14722,7 @@
         <v>276</v>
       </c>
       <c r="M11">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -14829,7 +14829,7 @@
         <v>83</v>
       </c>
       <c r="M2">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15157,7 +15157,7 @@
         <v>606</v>
       </c>
       <c r="M10">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15198,7 +15198,7 @@
         <v>1013</v>
       </c>
       <c r="M11">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -15766,7 +15766,7 @@
         <v>213</v>
       </c>
       <c r="M2">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -16094,7 +16094,7 @@
         <v>738</v>
       </c>
       <c r="M10">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16135,7 +16135,7 @@
         <v>1919</v>
       </c>
       <c r="M11">
-        <v>424</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -16715,7 +16715,7 @@
         <v>62</v>
       </c>
       <c r="M2">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -16940,7 +16940,7 @@
         <v>358</v>
       </c>
       <c r="M8">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17022,7 +17022,7 @@
         <v>1952</v>
       </c>
       <c r="M10">
-        <v>433</v>
+        <v>437</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17063,7 +17063,7 @@
         <v>2666</v>
       </c>
       <c r="M11">
-        <v>602</v>
+        <v>608</v>
       </c>
     </row>
   </sheetData>
@@ -17287,7 +17287,7 @@
         <v>82</v>
       </c>
       <c r="M5">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -17410,7 +17410,7 @@
         <v>209</v>
       </c>
       <c r="M8">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17492,7 +17492,7 @@
         <v>2708</v>
       </c>
       <c r="M10">
-        <v>527</v>
+        <v>534</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17533,7 +17533,7 @@
         <v>3351</v>
       </c>
       <c r="M11">
-        <v>666</v>
+        <v>677</v>
       </c>
     </row>
   </sheetData>
@@ -17681,7 +17681,7 @@
         <v>16</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -17856,7 +17856,7 @@
         <v>61</v>
       </c>
       <c r="M8">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17938,7 +17938,7 @@
         <v>302</v>
       </c>
       <c r="M10">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17979,7 +17979,7 @@
         <v>437</v>
       </c>
       <c r="M11">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -18370,7 +18370,7 @@
         <v>19</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -18452,7 +18452,7 @@
         <v>580</v>
       </c>
       <c r="M11">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -18824,7 +18824,7 @@
         <v>200</v>
       </c>
       <c r="M10">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -18865,7 +18865,7 @@
         <v>277</v>
       </c>
       <c r="M11">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -19255,7 +19255,7 @@
         <v>586</v>
       </c>
       <c r="M10">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19296,7 +19296,7 @@
         <v>745</v>
       </c>
       <c r="M11">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -19707,7 +19707,7 @@
         <v>1379</v>
       </c>
       <c r="M10">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19748,7 +19748,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>436</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>
@@ -20095,7 +20095,7 @@
         <v>324</v>
       </c>
       <c r="M8">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20177,7 +20177,7 @@
         <v>1108</v>
       </c>
       <c r="M10">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20218,7 +20218,7 @@
         <v>1719</v>
       </c>
       <c r="M11">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -20568,7 +20568,7 @@
         <v>251</v>
       </c>
       <c r="M8">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20650,7 +20650,7 @@
         <v>762</v>
       </c>
       <c r="M10">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20691,7 +20691,7 @@
         <v>1358</v>
       </c>
       <c r="M11">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -20918,7 +20918,7 @@
         <v>79</v>
       </c>
       <c r="M5">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -21123,7 +21123,7 @@
         <v>585</v>
       </c>
       <c r="M10">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21164,7 +21164,7 @@
         <v>1078</v>
       </c>
       <c r="M11">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -21514,7 +21514,7 @@
         <v>358</v>
       </c>
       <c r="M8">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21596,7 +21596,7 @@
         <v>2939</v>
       </c>
       <c r="M10">
-        <v>597</v>
+        <v>614</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21637,7 +21637,7 @@
         <v>3829</v>
       </c>
       <c r="M11">
-        <v>810</v>
+        <v>828</v>
       </c>
     </row>
   </sheetData>
@@ -21987,7 +21987,7 @@
         <v>206</v>
       </c>
       <c r="M8">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22069,7 +22069,7 @@
         <v>898</v>
       </c>
       <c r="M10">
-        <v>210</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22110,7 +22110,7 @@
         <v>1350</v>
       </c>
       <c r="M11">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -22463,7 +22463,7 @@
         <v>638</v>
       </c>
       <c r="M8">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22545,7 +22545,7 @@
         <v>1271</v>
       </c>
       <c r="M10">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22586,7 +22586,7 @@
         <v>3361</v>
       </c>
       <c r="M11">
-        <v>673</v>
+        <v>681</v>
       </c>
     </row>
   </sheetData>
@@ -22810,7 +22810,7 @@
         <v>206</v>
       </c>
       <c r="M5">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -23003,7 +23003,7 @@
         <v>2028</v>
       </c>
       <c r="M10">
-        <v>508</v>
+        <v>513</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23044,7 +23044,7 @@
         <v>2765</v>
       </c>
       <c r="M11">
-        <v>658</v>
+        <v>664</v>
       </c>
     </row>
   </sheetData>
@@ -23151,7 +23151,7 @@
         <v>211</v>
       </c>
       <c r="M2">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -23397,7 +23397,7 @@
         <v>410</v>
       </c>
       <c r="M8">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23479,7 +23479,7 @@
         <v>1124</v>
       </c>
       <c r="M10">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23520,7 +23520,7 @@
         <v>2329</v>
       </c>
       <c r="M11">
-        <v>473</v>
+        <v>481</v>
       </c>
     </row>
   </sheetData>
@@ -23919,7 +23919,7 @@
         <v>382</v>
       </c>
       <c r="M10">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23960,7 +23960,7 @@
         <v>601</v>
       </c>
       <c r="M11">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -24383,7 +24383,7 @@
         <v>592</v>
       </c>
       <c r="M10">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24424,7 +24424,7 @@
         <v>968</v>
       </c>
       <c r="M11">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -24572,7 +24572,7 @@
         <v>235</v>
       </c>
       <c r="M3">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -24695,7 +24695,7 @@
         <v>52</v>
       </c>
       <c r="M6">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -24777,7 +24777,7 @@
         <v>497</v>
       </c>
       <c r="M8">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24859,7 +24859,7 @@
         <v>1163</v>
       </c>
       <c r="M10">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24900,7 +24900,7 @@
         <v>2488</v>
       </c>
       <c r="M11">
-        <v>559</v>
+        <v>567</v>
       </c>
     </row>
   </sheetData>
@@ -25124,7 +25124,7 @@
         <v>29</v>
       </c>
       <c r="M5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -25229,7 +25229,7 @@
         <v>91</v>
       </c>
       <c r="M8">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -25308,7 +25308,7 @@
         <v>190</v>
       </c>
       <c r="M10">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25349,7 +25349,7 @@
         <v>386</v>
       </c>
       <c r="M11">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -25538,7 +25538,7 @@
         <v>14</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -25702,7 +25702,7 @@
         <v>571</v>
       </c>
       <c r="M8">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -25743,7 +25743,7 @@
         <v>165</v>
       </c>
       <c r="M9">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -25784,7 +25784,7 @@
         <v>938</v>
       </c>
       <c r="M10">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25825,7 +25825,7 @@
         <v>2409</v>
       </c>
       <c r="M11">
-        <v>441</v>
+        <v>446</v>
       </c>
     </row>
   </sheetData>
@@ -26169,7 +26169,7 @@
         <v>227</v>
       </c>
       <c r="M8">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -26251,7 +26251,7 @@
         <v>319</v>
       </c>
       <c r="M10">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26292,7 +26292,7 @@
         <v>778</v>
       </c>
       <c r="M11">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -26709,7 +26709,7 @@
         <v>168</v>
       </c>
       <c r="M10">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26750,7 +26750,7 @@
         <v>361</v>
       </c>
       <c r="M11">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -26857,7 +26857,7 @@
         <v>91</v>
       </c>
       <c r="M2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -27223,7 +27223,7 @@
         <v>1424</v>
       </c>
       <c r="M11">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>
@@ -27589,7 +27589,7 @@
         <v>204</v>
       </c>
       <c r="M10">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -27630,7 +27630,7 @@
         <v>266</v>
       </c>
       <c r="M11">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -27778,7 +27778,7 @@
         <v>39</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -27977,7 +27977,7 @@
         <v>122</v>
       </c>
       <c r="M8">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -28018,7 +28018,7 @@
         <v>41</v>
       </c>
       <c r="M9">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -28059,7 +28059,7 @@
         <v>824</v>
       </c>
       <c r="M10">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28100,7 +28100,7 @@
         <v>1154</v>
       </c>
       <c r="M11">
-        <v>294</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>
@@ -28248,7 +28248,7 @@
         <v>26</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -28493,7 +28493,7 @@
         <v>659</v>
       </c>
       <c r="M10">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28534,7 +28534,7 @@
         <v>902</v>
       </c>
       <c r="M11">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -28641,7 +28641,7 @@
         <v>75</v>
       </c>
       <c r="M2">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -28679,7 +28679,7 @@
         <v>84</v>
       </c>
       <c r="L3">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M3">
         <v>20</v>
@@ -28887,7 +28887,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -29007,10 +29007,10 @@
         <v>1939</v>
       </c>
       <c r="L11">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="M11">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -29415,7 +29415,7 @@
         <v>328</v>
       </c>
       <c r="M10">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29456,7 +29456,7 @@
         <v>500</v>
       </c>
       <c r="M11">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -30018,7 +30018,7 @@
         <v>70</v>
       </c>
       <c r="M2">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -30141,7 +30141,7 @@
         <v>73</v>
       </c>
       <c r="M5">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -30346,7 +30346,7 @@
         <v>424</v>
       </c>
       <c r="M10">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30387,7 +30387,7 @@
         <v>811</v>
       </c>
       <c r="M11">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -30535,7 +30535,7 @@
         <v>99</v>
       </c>
       <c r="M3">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -30655,7 +30655,7 @@
         <v>25</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -30775,7 +30775,7 @@
         <v>90</v>
       </c>
       <c r="M9">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -30816,7 +30816,7 @@
         <v>1041</v>
       </c>
       <c r="M10">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30857,7 +30857,7 @@
         <v>1776</v>
       </c>
       <c r="M11">
-        <v>439</v>
+        <v>443</v>
       </c>
     </row>
   </sheetData>
@@ -31078,7 +31078,7 @@
         <v>43</v>
       </c>
       <c r="M5">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -31283,7 +31283,7 @@
         <v>723</v>
       </c>
       <c r="M10">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31324,7 +31324,7 @@
         <v>1351</v>
       </c>
       <c r="M11">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -31554,7 +31554,7 @@
         <v>40</v>
       </c>
       <c r="M5">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -31677,7 +31677,7 @@
         <v>250</v>
       </c>
       <c r="M8">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -31759,7 +31759,7 @@
         <v>379</v>
       </c>
       <c r="M10">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31800,7 +31800,7 @@
         <v>966</v>
       </c>
       <c r="M11">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -31948,7 +31948,7 @@
         <v>79</v>
       </c>
       <c r="M3">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -32147,7 +32147,7 @@
         <v>309</v>
       </c>
       <c r="M8">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -32229,7 +32229,7 @@
         <v>813</v>
       </c>
       <c r="M10">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32270,7 +32270,7 @@
         <v>1445</v>
       </c>
       <c r="M11">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -32377,7 +32377,7 @@
         <v>171</v>
       </c>
       <c r="M2">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -32418,7 +32418,7 @@
         <v>190</v>
       </c>
       <c r="M3">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -32541,7 +32541,7 @@
         <v>49</v>
       </c>
       <c r="M6">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -32705,7 +32705,7 @@
         <v>729</v>
       </c>
       <c r="M10">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32746,7 +32746,7 @@
         <v>1695</v>
       </c>
       <c r="M11">
-        <v>368</v>
+        <v>374</v>
       </c>
     </row>
   </sheetData>
@@ -33585,7 +33585,7 @@
         <v>551</v>
       </c>
       <c r="M10">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33626,7 +33626,7 @@
         <v>939</v>
       </c>
       <c r="M11">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -34058,7 +34058,7 @@
         <v>480</v>
       </c>
       <c r="M10">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34099,7 +34099,7 @@
         <v>1090</v>
       </c>
       <c r="M11">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -34475,7 +34475,7 @@
         <v>29</v>
       </c>
       <c r="M9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -34516,7 +34516,7 @@
         <v>750</v>
       </c>
       <c r="M10">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34557,7 +34557,7 @@
         <v>1015</v>
       </c>
       <c r="M11">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -34784,7 +34784,7 @@
         <v>50</v>
       </c>
       <c r="M5">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -34898,7 +34898,7 @@
         <v>156</v>
       </c>
       <c r="M8">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -34980,7 +34980,7 @@
         <v>486</v>
       </c>
       <c r="M10">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35021,7 +35021,7 @@
         <v>803</v>
       </c>
       <c r="M11">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -35878,7 +35878,7 @@
         <v>527</v>
       </c>
       <c r="M10">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35919,7 +35919,7 @@
         <v>654</v>
       </c>
       <c r="M11">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -36146,7 +36146,7 @@
         <v>13</v>
       </c>
       <c r="M5">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -36269,7 +36269,7 @@
         <v>81</v>
       </c>
       <c r="M8">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -36392,7 +36392,7 @@
         <v>373</v>
       </c>
       <c r="M11">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -36758,7 +36758,7 @@
         <v>584</v>
       </c>
       <c r="M10">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36799,7 +36799,7 @@
         <v>620</v>
       </c>
       <c r="M11">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -37677,7 +37677,7 @@
         <v>532</v>
       </c>
       <c r="M10">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -37718,7 +37718,7 @@
         <v>924</v>
       </c>
       <c r="M11">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -38126,7 +38126,7 @@
         <v>449</v>
       </c>
       <c r="M10">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38167,7 +38167,7 @@
         <v>662</v>
       </c>
       <c r="M11">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -38566,7 +38566,7 @@
         <v>1036</v>
       </c>
       <c r="M10">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38607,7 +38607,7 @@
         <v>1460</v>
       </c>
       <c r="M11">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
   </sheetData>
@@ -39458,7 +39458,7 @@
         <v>408</v>
       </c>
       <c r="M10">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -39499,7 +39499,7 @@
         <v>597</v>
       </c>
       <c r="M11">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -39606,7 +39606,7 @@
         <v>11</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -39921,7 +39921,7 @@
         <v>470</v>
       </c>
       <c r="M11">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -40350,7 +40350,7 @@
         <v>386</v>
       </c>
       <c r="M10">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40391,7 +40391,7 @@
         <v>702</v>
       </c>
       <c r="M11">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -40539,7 +40539,7 @@
         <v>86</v>
       </c>
       <c r="M3">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -40820,7 +40820,7 @@
         <v>1430</v>
       </c>
       <c r="M10">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40861,7 +40861,7 @@
         <v>2036</v>
       </c>
       <c r="M11">
-        <v>379</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -41148,7 +41148,7 @@
         <v>26</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -41230,7 +41230,7 @@
         <v>265</v>
       </c>
       <c r="M10">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -41271,7 +41271,7 @@
         <v>322</v>
       </c>
       <c r="M11">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -41827,7 +41827,7 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -42066,7 +42066,7 @@
         <v>97</v>
       </c>
       <c r="M10">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -42107,7 +42107,7 @@
         <v>180</v>
       </c>
       <c r="M11">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -42311,6 +42311,9 @@
       <c r="K6">
         <v>1</v>
       </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
@@ -42478,7 +42481,7 @@
         <v>143</v>
       </c>
       <c r="M11">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -42804,7 +42807,7 @@
         <v>154</v>
       </c>
       <c r="M8">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -42845,7 +42848,7 @@
         <v>49</v>
       </c>
       <c r="M9">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -42886,7 +42889,7 @@
         <v>793</v>
       </c>
       <c r="M10">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -42927,7 +42930,7 @@
         <v>1128</v>
       </c>
       <c r="M11">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -43208,7 +43211,7 @@
         <v>35</v>
       </c>
       <c r="M8">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -43331,7 +43334,7 @@
         <v>237</v>
       </c>
       <c r="M11">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -44580,7 +44583,7 @@
         <v>152</v>
       </c>
       <c r="M10">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -44621,7 +44624,7 @@
         <v>231</v>
       </c>
       <c r="M11">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -45053,7 +45056,7 @@
         <v>168</v>
       </c>
       <c r="M10">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45094,7 +45097,7 @@
         <v>442</v>
       </c>
       <c r="M11">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -45201,7 +45204,7 @@
         <v>319</v>
       </c>
       <c r="M2">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -45242,7 +45245,7 @@
         <v>446</v>
       </c>
       <c r="M3">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -45324,7 +45327,7 @@
         <v>306</v>
       </c>
       <c r="M5">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -45365,7 +45368,7 @@
         <v>65</v>
       </c>
       <c r="M6">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -45447,7 +45450,7 @@
         <v>639</v>
       </c>
       <c r="M8">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45488,7 +45491,7 @@
         <v>226</v>
       </c>
       <c r="M9">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -45529,7 +45532,7 @@
         <v>1359</v>
       </c>
       <c r="M10">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45570,7 +45573,7 @@
         <v>3397</v>
       </c>
       <c r="M11">
-        <v>715</v>
+        <v>729</v>
       </c>
     </row>
   </sheetData>
@@ -45718,7 +45721,7 @@
         <v>16</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -46016,7 +46019,7 @@
         <v>298</v>
       </c>
       <c r="M11">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -46508,7 +46511,7 @@
         <v>25</v>
       </c>
       <c r="M2">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -46818,7 +46821,7 @@
         <v>294</v>
       </c>
       <c r="M10">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -46859,7 +46862,7 @@
         <v>467</v>
       </c>
       <c r="M11">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -46966,7 +46969,7 @@
         <v>67</v>
       </c>
       <c r="M2">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -47332,7 +47335,7 @@
         <v>874</v>
       </c>
       <c r="M11">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -48875,7 +48878,7 @@
         <v>93</v>
       </c>
       <c r="M9">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -48916,7 +48919,7 @@
         <v>134</v>
       </c>
       <c r="M10">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-08-03
</commit_message>
<xml_diff>
--- a/output/index-crime-full-year.xlsx
+++ b/output/index-crime-full-year.xlsx
@@ -913,7 +913,7 @@
         <v>6586</v>
       </c>
       <c r="M2">
-        <v>3698</v>
+        <v>3717</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -948,13 +948,13 @@
         <v>8085</v>
       </c>
       <c r="K3">
-        <v>8179</v>
+        <v>8178</v>
       </c>
       <c r="L3">
         <v>7116</v>
       </c>
       <c r="M3">
-        <v>4132</v>
+        <v>4152</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -995,7 +995,7 @@
         <v>374</v>
       </c>
       <c r="M4">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1036,7 +1036,7 @@
         <v>6212</v>
       </c>
       <c r="M5">
-        <v>3176</v>
+        <v>3199</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1056,10 +1056,10 @@
         <v>2075</v>
       </c>
       <c r="F6">
-        <v>1940</v>
+        <v>1941</v>
       </c>
       <c r="G6">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="H6">
         <v>1776</v>
@@ -1071,13 +1071,13 @@
         <v>1901</v>
       </c>
       <c r="K6">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="L6">
-        <v>1813</v>
+        <v>1812</v>
       </c>
       <c r="M6">
-        <v>1042</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1118,7 +1118,7 @@
         <v>433</v>
       </c>
       <c r="M7">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1159,7 +1159,7 @@
         <v>17250</v>
       </c>
       <c r="M8">
-        <v>10649</v>
+        <v>10689</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1200,7 +1200,7 @@
         <v>5809</v>
       </c>
       <c r="M9">
-        <v>2644</v>
+        <v>2671</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1241,7 +1241,7 @@
         <v>58700</v>
       </c>
       <c r="M10">
-        <v>33577</v>
+        <v>33722</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1261,10 +1261,10 @@
         <v>113478</v>
       </c>
       <c r="F11">
-        <v>105625</v>
+        <v>105626</v>
       </c>
       <c r="G11">
-        <v>85419</v>
+        <v>85420</v>
       </c>
       <c r="H11">
         <v>84717</v>
@@ -1279,10 +1279,10 @@
         <v>118787</v>
       </c>
       <c r="L11">
-        <v>104293</v>
+        <v>104292</v>
       </c>
       <c r="M11">
-        <v>59383</v>
+        <v>59665</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1389,7 @@
         <v>436</v>
       </c>
       <c r="M2">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1430,7 +1430,7 @@
         <v>504</v>
       </c>
       <c r="M3">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1512,7 +1512,7 @@
         <v>216</v>
       </c>
       <c r="M5">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1635,7 +1635,7 @@
         <v>777</v>
       </c>
       <c r="M8">
-        <v>510</v>
+        <v>511</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1676,7 +1676,7 @@
         <v>342</v>
       </c>
       <c r="M9">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1717,7 +1717,7 @@
         <v>1969</v>
       </c>
       <c r="M10">
-        <v>1095</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1758,7 +1758,7 @@
         <v>4423</v>
       </c>
       <c r="M11">
-        <v>2549</v>
+        <v>2558</v>
       </c>
     </row>
   </sheetData>
@@ -2274,7 +2274,7 @@
         <v>59</v>
       </c>
       <c r="M3">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2356,7 +2356,7 @@
         <v>91</v>
       </c>
       <c r="M5">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2379,7 +2379,7 @@
         <v>31</v>
       </c>
       <c r="G6">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H6">
         <v>26</v>
@@ -2476,7 +2476,7 @@
         <v>221</v>
       </c>
       <c r="M8">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2558,7 +2558,7 @@
         <v>1203</v>
       </c>
       <c r="M10">
-        <v>749</v>
+        <v>751</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2581,7 +2581,7 @@
         <v>1866</v>
       </c>
       <c r="G11">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="H11">
         <v>1184</v>
@@ -2599,7 +2599,7 @@
         <v>1756</v>
       </c>
       <c r="M11">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
   </sheetData>
@@ -2747,7 +2747,7 @@
         <v>446</v>
       </c>
       <c r="M3">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2788,7 +2788,7 @@
         <v>14</v>
       </c>
       <c r="M4">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2993,7 +2993,7 @@
         <v>226</v>
       </c>
       <c r="M9">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -3034,7 +3034,7 @@
         <v>1361</v>
       </c>
       <c r="M10">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3075,7 +3075,7 @@
         <v>3396</v>
       </c>
       <c r="M11">
-        <v>2013</v>
+        <v>2020</v>
       </c>
     </row>
   </sheetData>
@@ -3296,7 +3296,7 @@
         <v>28</v>
       </c>
       <c r="M5">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -3483,7 +3483,7 @@
         <v>338</v>
       </c>
       <c r="M10">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3524,7 +3524,7 @@
         <v>473</v>
       </c>
       <c r="M11">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -4089,7 +4089,7 @@
         <v>151</v>
       </c>
       <c r="M2">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -4130,7 +4130,7 @@
         <v>190</v>
       </c>
       <c r="M3">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4335,7 +4335,7 @@
         <v>377</v>
       </c>
       <c r="M8">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4376,7 +4376,7 @@
         <v>107</v>
       </c>
       <c r="M9">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4417,7 +4417,7 @@
         <v>493</v>
       </c>
       <c r="M10">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4458,7 +4458,7 @@
         <v>1486</v>
       </c>
       <c r="M11">
-        <v>850</v>
+        <v>856</v>
       </c>
     </row>
   </sheetData>
@@ -4606,7 +4606,7 @@
         <v>197</v>
       </c>
       <c r="M3">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4811,7 +4811,7 @@
         <v>468</v>
       </c>
       <c r="M8">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4852,7 +4852,7 @@
         <v>161</v>
       </c>
       <c r="M9">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4893,7 +4893,7 @@
         <v>863</v>
       </c>
       <c r="M10">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4934,7 +4934,7 @@
         <v>2090</v>
       </c>
       <c r="M11">
-        <v>1034</v>
+        <v>1039</v>
       </c>
     </row>
   </sheetData>
@@ -5082,7 +5082,7 @@
         <v>342</v>
       </c>
       <c r="M3">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5205,7 +5205,7 @@
         <v>71</v>
       </c>
       <c r="M6">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -5287,7 +5287,7 @@
         <v>460</v>
       </c>
       <c r="M8">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5328,7 +5328,7 @@
         <v>271</v>
       </c>
       <c r="M9">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5369,7 +5369,7 @@
         <v>876</v>
       </c>
       <c r="M10">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5410,7 +5410,7 @@
         <v>2444</v>
       </c>
       <c r="M11">
-        <v>1505</v>
+        <v>1516</v>
       </c>
     </row>
   </sheetData>
@@ -5558,7 +5558,7 @@
         <v>100</v>
       </c>
       <c r="M3">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5640,7 +5640,7 @@
         <v>147</v>
       </c>
       <c r="M5">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -5763,7 +5763,7 @@
         <v>285</v>
       </c>
       <c r="M8">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5845,7 +5845,7 @@
         <v>492</v>
       </c>
       <c r="M10">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5886,7 +5886,7 @@
         <v>1241</v>
       </c>
       <c r="M11">
-        <v>701</v>
+        <v>712</v>
       </c>
     </row>
   </sheetData>
@@ -6280,7 +6280,7 @@
         <v>79</v>
       </c>
       <c r="M9">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6321,7 +6321,7 @@
         <v>749</v>
       </c>
       <c r="M10">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6362,7 +6362,7 @@
         <v>1505</v>
       </c>
       <c r="M11">
-        <v>915</v>
+        <v>918</v>
       </c>
     </row>
   </sheetData>
@@ -6469,7 +6469,7 @@
         <v>928</v>
       </c>
       <c r="M2">
-        <v>493</v>
+        <v>496</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6633,7 +6633,7 @@
         <v>782</v>
       </c>
       <c r="M6">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -6674,7 +6674,7 @@
         <v>2412</v>
       </c>
       <c r="M7">
-        <v>1279</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6715,7 +6715,7 @@
         <v>4423</v>
       </c>
       <c r="M8">
-        <v>2549</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6756,7 +6756,7 @@
         <v>442</v>
       </c>
       <c r="M9">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6797,7 +6797,7 @@
         <v>1155</v>
       </c>
       <c r="M10">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6838,7 +6838,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>1136</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6961,7 +6961,7 @@
         <v>727</v>
       </c>
       <c r="M14">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -7043,7 +7043,7 @@
         <v>746</v>
       </c>
       <c r="M16">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7166,7 +7166,7 @@
         <v>2333</v>
       </c>
       <c r="M19">
-        <v>1238</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -7207,7 +7207,7 @@
         <v>1697</v>
       </c>
       <c r="M20">
-        <v>971</v>
+        <v>973</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -7248,7 +7248,7 @@
         <v>277</v>
       </c>
       <c r="M21">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -7330,7 +7330,7 @@
         <v>1353</v>
       </c>
       <c r="M23">
-        <v>745</v>
+        <v>752</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -7371,7 +7371,7 @@
         <v>533</v>
       </c>
       <c r="M24">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -7412,7 +7412,7 @@
         <v>580</v>
       </c>
       <c r="M25">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -7576,7 +7576,7 @@
         <v>3362</v>
       </c>
       <c r="M29">
-        <v>1889</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7617,7 +7617,7 @@
         <v>276</v>
       </c>
       <c r="M30">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -7658,7 +7658,7 @@
         <v>1015</v>
       </c>
       <c r="M31">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -7699,7 +7699,7 @@
         <v>180</v>
       </c>
       <c r="M32">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -7740,7 +7740,7 @@
         <v>2444</v>
       </c>
       <c r="M33">
-        <v>1505</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -7781,7 +7781,7 @@
         <v>702</v>
       </c>
       <c r="M34">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -7822,7 +7822,7 @@
         <v>322</v>
       </c>
       <c r="M35">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -7863,7 +7863,7 @@
         <v>1426</v>
       </c>
       <c r="M36">
-        <v>854</v>
+        <v>858</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7904,7 +7904,7 @@
         <v>2337</v>
       </c>
       <c r="M37">
-        <v>1334</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -7945,7 +7945,7 @@
         <v>134</v>
       </c>
       <c r="M38">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -7986,7 +7986,7 @@
         <v>181</v>
       </c>
       <c r="M39">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -8109,7 +8109,7 @@
         <v>2493</v>
       </c>
       <c r="M42">
-        <v>1817</v>
+        <v>1825</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -8150,7 +8150,7 @@
         <v>1461</v>
       </c>
       <c r="M43">
-        <v>675</v>
+        <v>679</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -8191,7 +8191,7 @@
         <v>972</v>
       </c>
       <c r="M44">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -8311,10 +8311,10 @@
         <v>1045</v>
       </c>
       <c r="L47">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="M47">
-        <v>558</v>
+        <v>561</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -8355,7 +8355,7 @@
         <v>2767</v>
       </c>
       <c r="M48">
-        <v>1632</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -8396,7 +8396,7 @@
         <v>1779</v>
       </c>
       <c r="M49">
-        <v>1057</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -8437,7 +8437,7 @@
         <v>1020</v>
       </c>
       <c r="M50">
-        <v>614</v>
+        <v>617</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -8478,7 +8478,7 @@
         <v>1445</v>
       </c>
       <c r="M51">
-        <v>882</v>
+        <v>883</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -8519,7 +8519,7 @@
         <v>1411</v>
       </c>
       <c r="M52">
-        <v>774</v>
+        <v>779</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -8542,7 +8542,7 @@
         <v>1866</v>
       </c>
       <c r="G53">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="H53">
         <v>1184</v>
@@ -8560,7 +8560,7 @@
         <v>1756</v>
       </c>
       <c r="M53">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -8601,7 +8601,7 @@
         <v>3832</v>
       </c>
       <c r="M54">
-        <v>2101</v>
+        <v>2107</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -8642,7 +8642,7 @@
         <v>1078</v>
       </c>
       <c r="M55">
-        <v>744</v>
+        <v>746</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -8683,7 +8683,7 @@
         <v>621</v>
       </c>
       <c r="M56">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -8724,7 +8724,7 @@
         <v>467</v>
       </c>
       <c r="M57">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -8765,7 +8765,7 @@
         <v>143</v>
       </c>
       <c r="M58">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -8847,7 +8847,7 @@
         <v>739</v>
       </c>
       <c r="M60">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -8888,7 +8888,7 @@
         <v>161</v>
       </c>
       <c r="M61">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -8949,7 +8949,7 @@
         <v>2128</v>
       </c>
       <c r="F63">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="G63">
         <v>1933</v>
@@ -8964,13 +8964,13 @@
         <v>1077</v>
       </c>
       <c r="K63">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="L63">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="M63">
-        <v>183</v>
+        <v>197</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -9011,7 +9011,7 @@
         <v>947</v>
       </c>
       <c r="M64">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -9052,7 +9052,7 @@
         <v>1385</v>
       </c>
       <c r="M65">
-        <v>804</v>
+        <v>805</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -9093,7 +9093,7 @@
         <v>602</v>
       </c>
       <c r="M66">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -9128,13 +9128,13 @@
         <v>2738</v>
       </c>
       <c r="K67">
-        <v>2433</v>
+        <v>2434</v>
       </c>
       <c r="L67">
-        <v>1921</v>
+        <v>1920</v>
       </c>
       <c r="M67">
-        <v>1151</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -9216,7 +9216,7 @@
         <v>473</v>
       </c>
       <c r="M69">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -9380,7 +9380,7 @@
         <v>1349</v>
       </c>
       <c r="M73">
-        <v>749</v>
+        <v>752</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -9421,7 +9421,7 @@
         <v>309</v>
       </c>
       <c r="M74">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -9503,7 +9503,7 @@
         <v>3354</v>
       </c>
       <c r="M76">
-        <v>1774</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -9544,7 +9544,7 @@
         <v>374</v>
       </c>
       <c r="M77">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -9585,7 +9585,7 @@
         <v>1583</v>
       </c>
       <c r="M78">
-        <v>690</v>
+        <v>693</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -9626,7 +9626,7 @@
         <v>2090</v>
       </c>
       <c r="M79">
-        <v>1034</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -9667,7 +9667,7 @@
         <v>470</v>
       </c>
       <c r="M80">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -9790,7 +9790,7 @@
         <v>1486</v>
       </c>
       <c r="M83">
-        <v>850</v>
+        <v>856</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -9831,7 +9831,7 @@
         <v>842</v>
       </c>
       <c r="M84">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="85" spans="1:13">
@@ -9872,7 +9872,7 @@
         <v>3396</v>
       </c>
       <c r="M85">
-        <v>2013</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -9913,7 +9913,7 @@
         <v>902</v>
       </c>
       <c r="M86">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -9954,7 +9954,7 @@
         <v>437</v>
       </c>
       <c r="M87">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -9995,7 +9995,7 @@
         <v>874</v>
       </c>
       <c r="M88">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -10036,7 +10036,7 @@
         <v>2036</v>
       </c>
       <c r="M89">
-        <v>1162</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -10077,7 +10077,7 @@
         <v>1089</v>
       </c>
       <c r="M90">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -10118,7 +10118,7 @@
         <v>968</v>
       </c>
       <c r="M91">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -10159,7 +10159,7 @@
         <v>316</v>
       </c>
       <c r="M92">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="93" spans="1:13">
@@ -10200,7 +10200,7 @@
         <v>803</v>
       </c>
       <c r="M93">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="94" spans="1:13">
@@ -10241,7 +10241,7 @@
         <v>2670</v>
       </c>
       <c r="M94">
-        <v>1631</v>
+        <v>1638</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -10282,7 +10282,7 @@
         <v>1241</v>
       </c>
       <c r="M95">
-        <v>701</v>
+        <v>712</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -10323,7 +10323,7 @@
         <v>1361</v>
       </c>
       <c r="M96">
-        <v>636</v>
+        <v>641</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -10364,7 +10364,7 @@
         <v>1719</v>
       </c>
       <c r="M97">
-        <v>906</v>
+        <v>907</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -10446,7 +10446,7 @@
         <v>1505</v>
       </c>
       <c r="M99">
-        <v>915</v>
+        <v>918</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -10487,7 +10487,7 @@
         <v>277</v>
       </c>
       <c r="M100">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="101" spans="1:13">
@@ -10507,10 +10507,10 @@
         <v>113478</v>
       </c>
       <c r="F101">
-        <v>105625</v>
+        <v>105626</v>
       </c>
       <c r="G101">
-        <v>85419</v>
+        <v>85420</v>
       </c>
       <c r="H101">
         <v>84717</v>
@@ -10525,10 +10525,10 @@
         <v>118787</v>
       </c>
       <c r="L101">
-        <v>104293</v>
+        <v>104292</v>
       </c>
       <c r="M101">
-        <v>59383</v>
+        <v>59665</v>
       </c>
     </row>
   </sheetData>
@@ -10778,7 +10778,7 @@
         <v>22</v>
       </c>
       <c r="M3">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -10968,7 +10968,7 @@
         <v>59</v>
       </c>
       <c r="M8">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11091,7 +11091,7 @@
         <v>276</v>
       </c>
       <c r="M11">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -11356,10 +11356,10 @@
         <v>72</v>
       </c>
       <c r="K6">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L6">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="M6">
         <v>29</v>
@@ -11444,7 +11444,7 @@
         <v>319</v>
       </c>
       <c r="M8">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11485,7 +11485,7 @@
         <v>177</v>
       </c>
       <c r="M9">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -11526,7 +11526,7 @@
         <v>740</v>
       </c>
       <c r="M10">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -11561,13 +11561,13 @@
         <v>2738</v>
       </c>
       <c r="K11">
-        <v>2433</v>
+        <v>2434</v>
       </c>
       <c r="L11">
-        <v>1921</v>
+        <v>1920</v>
       </c>
       <c r="M11">
-        <v>1151</v>
+        <v>1158</v>
       </c>
     </row>
   </sheetData>
@@ -12002,7 +12002,7 @@
         <v>606</v>
       </c>
       <c r="M10">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12043,7 +12043,7 @@
         <v>1015</v>
       </c>
       <c r="M11">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
   </sheetData>
@@ -12478,7 +12478,7 @@
         <v>399</v>
       </c>
       <c r="M10">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12519,7 +12519,7 @@
         <v>842</v>
       </c>
       <c r="M11">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -12667,7 +12667,7 @@
         <v>137</v>
       </c>
       <c r="M3">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -12995,7 +12995,7 @@
         <v>1385</v>
       </c>
       <c r="M11">
-        <v>804</v>
+        <v>805</v>
       </c>
     </row>
   </sheetData>
@@ -13566,7 +13566,7 @@
         <v>250</v>
       </c>
       <c r="M2">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -13689,7 +13689,7 @@
         <v>171</v>
       </c>
       <c r="M5">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13730,7 +13730,7 @@
         <v>52</v>
       </c>
       <c r="M6">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -13853,7 +13853,7 @@
         <v>210</v>
       </c>
       <c r="M9">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -13894,7 +13894,7 @@
         <v>902</v>
       </c>
       <c r="M10">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13935,7 +13935,7 @@
         <v>2337</v>
       </c>
       <c r="M11">
-        <v>1334</v>
+        <v>1340</v>
       </c>
     </row>
   </sheetData>
@@ -15057,7 +15057,7 @@
         <v>42</v>
       </c>
       <c r="M5">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -15262,7 +15262,7 @@
         <v>447</v>
       </c>
       <c r="M10">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15303,7 +15303,7 @@
         <v>739</v>
       </c>
       <c r="M11">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -15410,7 +15410,7 @@
         <v>244</v>
       </c>
       <c r="M2">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15451,7 +15451,7 @@
         <v>220</v>
       </c>
       <c r="M3">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -15697,7 +15697,7 @@
         <v>166</v>
       </c>
       <c r="M9">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -15738,7 +15738,7 @@
         <v>939</v>
       </c>
       <c r="M10">
-        <v>573</v>
+        <v>576</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15779,7 +15779,7 @@
         <v>2412</v>
       </c>
       <c r="M11">
-        <v>1279</v>
+        <v>1285</v>
       </c>
     </row>
   </sheetData>
@@ -16117,7 +16117,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16199,7 +16199,7 @@
         <v>544</v>
       </c>
       <c r="M10">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16240,7 +16240,7 @@
         <v>947</v>
       </c>
       <c r="M11">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>
@@ -17009,7 +17009,7 @@
         <v>360</v>
       </c>
       <c r="M8">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17091,7 +17091,7 @@
         <v>1953</v>
       </c>
       <c r="M10">
-        <v>1171</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17132,7 +17132,7 @@
         <v>2670</v>
       </c>
       <c r="M11">
-        <v>1631</v>
+        <v>1638</v>
       </c>
     </row>
   </sheetData>
@@ -17479,7 +17479,7 @@
         <v>208</v>
       </c>
       <c r="M8">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17520,7 +17520,7 @@
         <v>161</v>
       </c>
       <c r="M9">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -17561,7 +17561,7 @@
         <v>2711</v>
       </c>
       <c r="M10">
-        <v>1403</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17602,7 +17602,7 @@
         <v>3354</v>
       </c>
       <c r="M11">
-        <v>1774</v>
+        <v>1785</v>
       </c>
     </row>
   </sheetData>
@@ -17928,7 +17928,7 @@
         <v>61</v>
       </c>
       <c r="M8">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -18051,7 +18051,7 @@
         <v>437</v>
       </c>
       <c r="M11">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>
@@ -18344,7 +18344,7 @@
         <v>18</v>
       </c>
       <c r="M8">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -18426,7 +18426,7 @@
         <v>200</v>
       </c>
       <c r="M10">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -18467,7 +18467,7 @@
         <v>277</v>
       </c>
       <c r="M11">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -18574,7 +18574,7 @@
         <v>42</v>
       </c>
       <c r="M2">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -18899,7 +18899,7 @@
         <v>218</v>
       </c>
       <c r="M10">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -18940,7 +18940,7 @@
         <v>580</v>
       </c>
       <c r="M11">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -19149,7 +19149,7 @@
         <v>48</v>
       </c>
       <c r="M5">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -19333,7 +19333,7 @@
         <v>587</v>
       </c>
       <c r="M10">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19374,7 +19374,7 @@
         <v>746</v>
       </c>
       <c r="M11">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -19791,7 +19791,7 @@
         <v>1379</v>
       </c>
       <c r="M10">
-        <v>788</v>
+        <v>789</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19832,7 +19832,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>1057</v>
+        <v>1058</v>
       </c>
     </row>
   </sheetData>
@@ -20261,7 +20261,7 @@
         <v>1107</v>
       </c>
       <c r="M10">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20302,7 +20302,7 @@
         <v>1719</v>
       </c>
       <c r="M11">
-        <v>906</v>
+        <v>907</v>
       </c>
     </row>
   </sheetData>
@@ -20643,7 +20643,7 @@
         <v>121</v>
       </c>
       <c r="M8">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20725,7 +20725,7 @@
         <v>427</v>
       </c>
       <c r="M10">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20766,7 +20766,7 @@
         <v>727</v>
       </c>
       <c r="M11">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -20873,7 +20873,7 @@
         <v>65</v>
       </c>
       <c r="M2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20914,7 +20914,7 @@
         <v>75</v>
       </c>
       <c r="M3">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -21242,7 +21242,7 @@
         <v>1078</v>
       </c>
       <c r="M11">
-        <v>744</v>
+        <v>746</v>
       </c>
     </row>
   </sheetData>
@@ -21633,7 +21633,7 @@
         <v>207</v>
       </c>
       <c r="M9">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -21674,7 +21674,7 @@
         <v>2940</v>
       </c>
       <c r="M10">
-        <v>1598</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21715,7 +21715,7 @@
         <v>3832</v>
       </c>
       <c r="M11">
-        <v>2101</v>
+        <v>2107</v>
       </c>
     </row>
   </sheetData>
@@ -21822,7 +21822,7 @@
         <v>61</v>
       </c>
       <c r="M2">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -22147,7 +22147,7 @@
         <v>898</v>
       </c>
       <c r="M10">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22188,7 +22188,7 @@
         <v>1349</v>
       </c>
       <c r="M11">
-        <v>749</v>
+        <v>752</v>
       </c>
     </row>
   </sheetData>
@@ -22295,7 +22295,7 @@
         <v>370</v>
       </c>
       <c r="M2">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -22500,7 +22500,7 @@
         <v>21</v>
       </c>
       <c r="M7">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -22541,7 +22541,7 @@
         <v>639</v>
       </c>
       <c r="M8">
-        <v>407</v>
+        <v>413</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22582,7 +22582,7 @@
         <v>287</v>
       </c>
       <c r="M9">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -22623,7 +22623,7 @@
         <v>1271</v>
       </c>
       <c r="M10">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22664,7 +22664,7 @@
         <v>3362</v>
       </c>
       <c r="M11">
-        <v>1889</v>
+        <v>1902</v>
       </c>
     </row>
   </sheetData>
@@ -23017,7 +23017,7 @@
         <v>410</v>
       </c>
       <c r="M8">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23140,7 +23140,7 @@
         <v>2333</v>
       </c>
       <c r="M11">
-        <v>1238</v>
+        <v>1240</v>
       </c>
     </row>
   </sheetData>
@@ -23539,7 +23539,7 @@
         <v>383</v>
       </c>
       <c r="M10">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23580,7 +23580,7 @@
         <v>602</v>
       </c>
       <c r="M11">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -24458,7 +24458,7 @@
         <v>596</v>
       </c>
       <c r="M10">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24499,7 +24499,7 @@
         <v>972</v>
       </c>
       <c r="M11">
-        <v>586</v>
+        <v>589</v>
       </c>
     </row>
   </sheetData>
@@ -24606,7 +24606,7 @@
         <v>187</v>
       </c>
       <c r="M2">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -24647,7 +24647,7 @@
         <v>235</v>
       </c>
       <c r="M3">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -24729,7 +24729,7 @@
         <v>136</v>
       </c>
       <c r="M5">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -24852,7 +24852,7 @@
         <v>497</v>
       </c>
       <c r="M8">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24893,7 +24893,7 @@
         <v>190</v>
       </c>
       <c r="M9">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -24934,7 +24934,7 @@
         <v>1167</v>
       </c>
       <c r="M10">
-        <v>907</v>
+        <v>909</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24975,7 +24975,7 @@
         <v>2493</v>
       </c>
       <c r="M11">
-        <v>1817</v>
+        <v>1825</v>
       </c>
     </row>
   </sheetData>
@@ -25123,7 +25123,7 @@
         <v>69</v>
       </c>
       <c r="M3">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -25199,7 +25199,7 @@
         <v>206</v>
       </c>
       <c r="M5">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -25240,7 +25240,7 @@
         <v>56</v>
       </c>
       <c r="M6">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -25310,7 +25310,7 @@
         <v>251</v>
       </c>
       <c r="M8">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -25392,7 +25392,7 @@
         <v>2032</v>
       </c>
       <c r="M10">
-        <v>1270</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25433,7 +25433,7 @@
         <v>2767</v>
       </c>
       <c r="M11">
-        <v>1632</v>
+        <v>1641</v>
       </c>
     </row>
   </sheetData>
@@ -26208,7 +26208,7 @@
         <v>227</v>
       </c>
       <c r="M8">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -26249,7 +26249,7 @@
         <v>34</v>
       </c>
       <c r="M9">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -26290,7 +26290,7 @@
         <v>321</v>
       </c>
       <c r="M10">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26331,7 +26331,7 @@
         <v>782</v>
       </c>
       <c r="M11">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
   </sheetData>
@@ -26902,7 +26902,7 @@
         <v>92</v>
       </c>
       <c r="M2">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -27145,7 +27145,7 @@
         <v>438</v>
       </c>
       <c r="M8">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -27227,7 +27227,7 @@
         <v>638</v>
       </c>
       <c r="M10">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -27268,7 +27268,7 @@
         <v>1426</v>
       </c>
       <c r="M11">
-        <v>854</v>
+        <v>858</v>
       </c>
     </row>
   </sheetData>
@@ -28116,7 +28116,7 @@
         <v>824</v>
       </c>
       <c r="M10">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28157,7 +28157,7 @@
         <v>1155</v>
       </c>
       <c r="M11">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
   </sheetData>
@@ -28407,7 +28407,7 @@
         <v>71</v>
       </c>
       <c r="M6">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -28591,7 +28591,7 @@
         <v>902</v>
       </c>
       <c r="M11">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
   </sheetData>
@@ -28985,7 +28985,7 @@
         <v>82</v>
       </c>
       <c r="M9">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -29026,7 +29026,7 @@
         <v>976</v>
       </c>
       <c r="M10">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29067,7 +29067,7 @@
         <v>1583</v>
       </c>
       <c r="M11">
-        <v>690</v>
+        <v>693</v>
       </c>
     </row>
   </sheetData>
@@ -30409,7 +30409,7 @@
         <v>307</v>
       </c>
       <c r="M10">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30450,7 +30450,7 @@
         <v>533</v>
       </c>
       <c r="M11">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -30598,7 +30598,7 @@
         <v>69</v>
       </c>
       <c r="M3">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -30680,7 +30680,7 @@
         <v>104</v>
       </c>
       <c r="M5">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -30844,7 +30844,7 @@
         <v>67</v>
       </c>
       <c r="M9">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -30885,7 +30885,7 @@
         <v>763</v>
       </c>
       <c r="M10">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30926,7 +30926,7 @@
         <v>1361</v>
       </c>
       <c r="M11">
-        <v>636</v>
+        <v>641</v>
       </c>
     </row>
   </sheetData>
@@ -31270,7 +31270,7 @@
         <v>354</v>
       </c>
       <c r="M8">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -31311,7 +31311,7 @@
         <v>59</v>
       </c>
       <c r="M9">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -31352,7 +31352,7 @@
         <v>725</v>
       </c>
       <c r="M10">
-        <v>387</v>
+        <v>391</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31393,7 +31393,7 @@
         <v>1353</v>
       </c>
       <c r="M11">
-        <v>745</v>
+        <v>752</v>
       </c>
     </row>
   </sheetData>
@@ -31740,7 +31740,7 @@
         <v>309</v>
       </c>
       <c r="M8">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -31863,7 +31863,7 @@
         <v>1445</v>
       </c>
       <c r="M11">
-        <v>882</v>
+        <v>883</v>
       </c>
     </row>
   </sheetData>
@@ -32298,7 +32298,7 @@
         <v>730</v>
       </c>
       <c r="M10">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32339,7 +32339,7 @@
         <v>1697</v>
       </c>
       <c r="M11">
-        <v>971</v>
+        <v>973</v>
       </c>
     </row>
   </sheetData>
@@ -32569,7 +32569,7 @@
         <v>40</v>
       </c>
       <c r="M5">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -32815,7 +32815,7 @@
         <v>968</v>
       </c>
       <c r="M11">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
   </sheetData>
@@ -33196,7 +33196,7 @@
         <v>168</v>
       </c>
       <c r="M10">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33237,7 +33237,7 @@
         <v>277</v>
       </c>
       <c r="M11">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>
@@ -33458,7 +33458,7 @@
         <v>49</v>
       </c>
       <c r="L5">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M5">
         <v>29</v>
@@ -33660,7 +33660,7 @@
         <v>552</v>
       </c>
       <c r="M10">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33698,10 +33698,10 @@
         <v>1045</v>
       </c>
       <c r="L11">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="M11">
-        <v>558</v>
+        <v>561</v>
       </c>
     </row>
   </sheetData>
@@ -34054,7 +34054,7 @@
         <v>294</v>
       </c>
       <c r="M8">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -34095,7 +34095,7 @@
         <v>62</v>
       </c>
       <c r="M9">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -34136,7 +34136,7 @@
         <v>480</v>
       </c>
       <c r="M10">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34177,7 +34177,7 @@
         <v>1089</v>
       </c>
       <c r="M11">
-        <v>506</v>
+        <v>510</v>
       </c>
     </row>
   </sheetData>
@@ -34398,7 +34398,7 @@
         <v>64</v>
       </c>
       <c r="M5">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -34597,7 +34597,7 @@
         <v>750</v>
       </c>
       <c r="M10">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34638,7 +34638,7 @@
         <v>1020</v>
       </c>
       <c r="M11">
-        <v>614</v>
+        <v>617</v>
       </c>
     </row>
   </sheetData>
@@ -35061,7 +35061,7 @@
         <v>486</v>
       </c>
       <c r="M10">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35102,7 +35102,7 @@
         <v>803</v>
       </c>
       <c r="M11">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -35849,7 +35849,7 @@
         <v>44</v>
       </c>
       <c r="M6">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -36010,7 +36010,7 @@
         <v>1425</v>
       </c>
       <c r="M10">
-        <v>841</v>
+        <v>851</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36051,7 +36051,7 @@
         <v>2036</v>
       </c>
       <c r="M11">
-        <v>1162</v>
+        <v>1173</v>
       </c>
     </row>
   </sheetData>
@@ -36278,7 +36278,7 @@
         <v>13</v>
       </c>
       <c r="M5">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -36524,7 +36524,7 @@
         <v>374</v>
       </c>
       <c r="M11">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -36902,7 +36902,7 @@
         <v>584</v>
       </c>
       <c r="M10">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36943,7 +36943,7 @@
         <v>621</v>
       </c>
       <c r="M11">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -37496,7 +37496,7 @@
         <v>63</v>
       </c>
       <c r="M2">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -37824,7 +37824,7 @@
         <v>533</v>
       </c>
       <c r="M10">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -37865,7 +37865,7 @@
         <v>928</v>
       </c>
       <c r="M11">
-        <v>493</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>
@@ -38468,7 +38468,7 @@
         <v>57</v>
       </c>
       <c r="M3">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -38532,7 +38532,7 @@
         <v>70</v>
       </c>
       <c r="M5">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -38684,7 +38684,7 @@
         <v>49</v>
       </c>
       <c r="M9">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -38766,7 +38766,7 @@
         <v>1461</v>
       </c>
       <c r="M11">
-        <v>675</v>
+        <v>679</v>
       </c>
     </row>
   </sheetData>
@@ -40042,7 +40042,7 @@
         <v>366</v>
       </c>
       <c r="M10">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40083,7 +40083,7 @@
         <v>470</v>
       </c>
       <c r="M11">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -40515,7 +40515,7 @@
         <v>386</v>
       </c>
       <c r="M10">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40556,7 +40556,7 @@
         <v>702</v>
       </c>
       <c r="M11">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
   </sheetData>
@@ -40663,7 +40663,7 @@
         <v>133</v>
       </c>
       <c r="M2">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -40947,7 +40947,7 @@
         <v>90</v>
       </c>
       <c r="M9">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -40988,7 +40988,7 @@
         <v>1041</v>
       </c>
       <c r="M10">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -41029,7 +41029,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>1136</v>
+        <v>1140</v>
       </c>
     </row>
   </sheetData>
@@ -41360,7 +41360,7 @@
         <v>12</v>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -41442,7 +41442,7 @@
         <v>322</v>
       </c>
       <c r="M11">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -41651,7 +41651,7 @@
         <v>14</v>
       </c>
       <c r="M5">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -41832,7 +41832,7 @@
         <v>97</v>
       </c>
       <c r="M10">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -41873,7 +41873,7 @@
         <v>180</v>
       </c>
       <c r="M11">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -42875,7 +42875,7 @@
         <v>4</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -43037,7 +43037,7 @@
         <v>4</v>
       </c>
       <c r="M9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -43119,7 +43119,7 @@
         <v>143</v>
       </c>
       <c r="M11">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -43955,7 +43955,7 @@
         <v>151</v>
       </c>
       <c r="M10">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -43996,7 +43996,7 @@
         <v>316</v>
       </c>
       <c r="M11">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -44103,7 +44103,7 @@
         <v>6</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -44202,7 +44202,7 @@
         <v>15</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -44368,7 +44368,7 @@
         <v>98</v>
       </c>
       <c r="M10">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -44409,7 +44409,7 @@
         <v>161</v>
       </c>
       <c r="M11">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -45266,7 +45266,7 @@
         <v>168</v>
       </c>
       <c r="M10">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45307,7 +45307,7 @@
         <v>442</v>
       </c>
       <c r="M11">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -45414,7 +45414,7 @@
         <v>145</v>
       </c>
       <c r="M2">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -45537,7 +45537,7 @@
         <v>80</v>
       </c>
       <c r="M5">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -45660,7 +45660,7 @@
         <v>184</v>
       </c>
       <c r="M8">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45742,7 +45742,7 @@
         <v>683</v>
       </c>
       <c r="M10">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45783,7 +45783,7 @@
         <v>1411</v>
       </c>
       <c r="M11">
-        <v>774</v>
+        <v>779</v>
       </c>
     </row>
   </sheetData>
@@ -46573,7 +46573,7 @@
         <v>146</v>
       </c>
       <c r="M8">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -46614,7 +46614,7 @@
         <v>181</v>
       </c>
       <c r="M9">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -47034,7 +47034,7 @@
         <v>294</v>
       </c>
       <c r="M10">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -47075,7 +47075,7 @@
         <v>467</v>
       </c>
       <c r="M11">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>
@@ -47182,7 +47182,7 @@
         <v>67</v>
       </c>
       <c r="M2">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -47223,7 +47223,7 @@
         <v>75</v>
       </c>
       <c r="M3">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -47551,7 +47551,7 @@
         <v>874</v>
       </c>
       <c r="M11">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
   </sheetData>
@@ -47923,7 +47923,7 @@
         <v>264</v>
       </c>
       <c r="M10">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -47964,7 +47964,7 @@
         <v>309</v>
       </c>
       <c r="M11">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -49038,7 +49038,7 @@
         <v>14</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -49079,7 +49079,7 @@
         <v>7</v>
       </c>
       <c r="M9">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -49161,7 +49161,7 @@
         <v>134</v>
       </c>
       <c r="M11">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-08-17
</commit_message>
<xml_diff>
--- a/output/index-crime-full-year.xlsx
+++ b/output/index-crime-full-year.xlsx
@@ -913,7 +913,7 @@
         <v>6587</v>
       </c>
       <c r="M2">
-        <v>3940</v>
+        <v>3964</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -954,7 +954,7 @@
         <v>7117</v>
       </c>
       <c r="M3">
-        <v>4432</v>
+        <v>4461</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -995,7 +995,7 @@
         <v>374</v>
       </c>
       <c r="M4">
-        <v>224</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1036,7 +1036,7 @@
         <v>6211</v>
       </c>
       <c r="M5">
-        <v>3422</v>
+        <v>3440</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1077,7 +1077,7 @@
         <v>1815</v>
       </c>
       <c r="M6">
-        <v>1115</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1118,7 +1118,7 @@
         <v>433</v>
       </c>
       <c r="M7">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1159,7 +1159,7 @@
         <v>17253</v>
       </c>
       <c r="M8">
-        <v>11387</v>
+        <v>11459</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1200,7 +1200,7 @@
         <v>5809</v>
       </c>
       <c r="M9">
-        <v>2902</v>
+        <v>2918</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1241,7 +1241,7 @@
         <v>58706</v>
       </c>
       <c r="M10">
-        <v>35489</v>
+        <v>35599</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1282,7 +1282,7 @@
         <v>104305</v>
       </c>
       <c r="M11">
-        <v>63178</v>
+        <v>63464</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1389,7 @@
         <v>436</v>
       </c>
       <c r="M2">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1430,7 +1430,7 @@
         <v>504</v>
       </c>
       <c r="M3">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1635,7 +1635,7 @@
         <v>777</v>
       </c>
       <c r="M8">
-        <v>556</v>
+        <v>560</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1717,7 +1717,7 @@
         <v>1969</v>
       </c>
       <c r="M10">
-        <v>1163</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1758,7 +1758,7 @@
         <v>4423</v>
       </c>
       <c r="M11">
-        <v>2740</v>
+        <v>2753</v>
       </c>
     </row>
   </sheetData>
@@ -2044,7 +2044,7 @@
         <v>3</v>
       </c>
       <c r="M9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2126,7 +2126,7 @@
         <v>61</v>
       </c>
       <c r="M11">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2274,7 +2274,7 @@
         <v>59</v>
       </c>
       <c r="M3">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2476,7 +2476,7 @@
         <v>221</v>
       </c>
       <c r="M8">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2558,7 +2558,7 @@
         <v>1203</v>
       </c>
       <c r="M10">
-        <v>785</v>
+        <v>790</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2599,7 +2599,7 @@
         <v>1756</v>
       </c>
       <c r="M11">
-        <v>1117</v>
+        <v>1125</v>
       </c>
     </row>
   </sheetData>
@@ -2747,7 +2747,7 @@
         <v>446</v>
       </c>
       <c r="M3">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2829,7 +2829,7 @@
         <v>304</v>
       </c>
       <c r="M5">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2952,7 +2952,7 @@
         <v>637</v>
       </c>
       <c r="M8">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3034,7 +3034,7 @@
         <v>1361</v>
       </c>
       <c r="M10">
-        <v>860</v>
+        <v>863</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3075,7 +3075,7 @@
         <v>3396</v>
       </c>
       <c r="M11">
-        <v>2147</v>
+        <v>2160</v>
       </c>
     </row>
   </sheetData>
@@ -3401,7 +3401,7 @@
         <v>58</v>
       </c>
       <c r="M8">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3483,7 +3483,7 @@
         <v>338</v>
       </c>
       <c r="M10">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3524,7 +3524,7 @@
         <v>473</v>
       </c>
       <c r="M11">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -3786,7 +3786,7 @@
         <v>9</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3859,7 +3859,7 @@
         <v>64</v>
       </c>
       <c r="M8">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3941,7 +3941,7 @@
         <v>265</v>
       </c>
       <c r="M10">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3982,7 +3982,7 @@
         <v>427</v>
       </c>
       <c r="M11">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -4089,7 +4089,7 @@
         <v>151</v>
       </c>
       <c r="M2">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -4130,7 +4130,7 @@
         <v>190</v>
       </c>
       <c r="M3">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4335,7 +4335,7 @@
         <v>377</v>
       </c>
       <c r="M8">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4417,7 +4417,7 @@
         <v>493</v>
       </c>
       <c r="M10">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4458,7 +4458,7 @@
         <v>1486</v>
       </c>
       <c r="M11">
-        <v>916</v>
+        <v>920</v>
       </c>
     </row>
   </sheetData>
@@ -4606,7 +4606,7 @@
         <v>197</v>
       </c>
       <c r="M3">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4729,7 +4729,7 @@
         <v>39</v>
       </c>
       <c r="M6">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -4893,7 +4893,7 @@
         <v>863</v>
       </c>
       <c r="M10">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4934,7 +4934,7 @@
         <v>2091</v>
       </c>
       <c r="M11">
-        <v>1109</v>
+        <v>1112</v>
       </c>
     </row>
   </sheetData>
@@ -5082,7 +5082,7 @@
         <v>342</v>
       </c>
       <c r="M3">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5246,7 +5246,7 @@
         <v>25</v>
       </c>
       <c r="M7">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -5287,7 +5287,7 @@
         <v>460</v>
       </c>
       <c r="M8">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5369,7 +5369,7 @@
         <v>876</v>
       </c>
       <c r="M10">
-        <v>614</v>
+        <v>617</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5410,7 +5410,7 @@
         <v>2444</v>
       </c>
       <c r="M11">
-        <v>1615</v>
+        <v>1621</v>
       </c>
     </row>
   </sheetData>
@@ -5558,7 +5558,7 @@
         <v>100</v>
       </c>
       <c r="M3">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5599,7 +5599,7 @@
         <v>15</v>
       </c>
       <c r="M4">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -5763,7 +5763,7 @@
         <v>285</v>
       </c>
       <c r="M8">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5804,7 +5804,7 @@
         <v>70</v>
       </c>
       <c r="M9">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5845,7 +5845,7 @@
         <v>492</v>
       </c>
       <c r="M10">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5886,7 +5886,7 @@
         <v>1241</v>
       </c>
       <c r="M11">
-        <v>761</v>
+        <v>766</v>
       </c>
     </row>
   </sheetData>
@@ -6321,7 +6321,7 @@
         <v>749</v>
       </c>
       <c r="M10">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6362,7 +6362,7 @@
         <v>1505</v>
       </c>
       <c r="M11">
-        <v>980</v>
+        <v>983</v>
       </c>
     </row>
   </sheetData>
@@ -6469,7 +6469,7 @@
         <v>928</v>
       </c>
       <c r="M2">
-        <v>524</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6551,7 +6551,7 @@
         <v>597</v>
       </c>
       <c r="M4">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6592,7 +6592,7 @@
         <v>266</v>
       </c>
       <c r="M5">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -6633,7 +6633,7 @@
         <v>782</v>
       </c>
       <c r="M6">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -6674,7 +6674,7 @@
         <v>2412</v>
       </c>
       <c r="M7">
-        <v>1388</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6715,7 +6715,7 @@
         <v>4423</v>
       </c>
       <c r="M8">
-        <v>2740</v>
+        <v>2753</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6797,7 +6797,7 @@
         <v>1155</v>
       </c>
       <c r="M10">
-        <v>746</v>
+        <v>749</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6838,7 +6838,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>1196</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6879,7 +6879,7 @@
         <v>414</v>
       </c>
       <c r="M12">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -6920,7 +6920,7 @@
         <v>267</v>
       </c>
       <c r="M13">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -6961,7 +6961,7 @@
         <v>727</v>
       </c>
       <c r="M14">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -7002,7 +7002,7 @@
         <v>813</v>
       </c>
       <c r="M15">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -7043,7 +7043,7 @@
         <v>746</v>
       </c>
       <c r="M16">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -7084,7 +7084,7 @@
         <v>128</v>
       </c>
       <c r="M17">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -7125,7 +7125,7 @@
         <v>642</v>
       </c>
       <c r="M18">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -7166,7 +7166,7 @@
         <v>2333</v>
       </c>
       <c r="M19">
-        <v>1311</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -7207,7 +7207,7 @@
         <v>1697</v>
       </c>
       <c r="M20">
-        <v>1018</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -7248,7 +7248,7 @@
         <v>277</v>
       </c>
       <c r="M21">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -7289,7 +7289,7 @@
         <v>385</v>
       </c>
       <c r="M22">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -7330,7 +7330,7 @@
         <v>1353</v>
       </c>
       <c r="M23">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -7371,7 +7371,7 @@
         <v>533</v>
       </c>
       <c r="M24">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -7412,7 +7412,7 @@
         <v>580</v>
       </c>
       <c r="M25">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -7494,7 +7494,7 @@
         <v>1242</v>
       </c>
       <c r="M27">
-        <v>698</v>
+        <v>701</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -7576,7 +7576,7 @@
         <v>3362</v>
       </c>
       <c r="M29">
-        <v>2038</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7658,7 +7658,7 @@
         <v>1015</v>
       </c>
       <c r="M31">
-        <v>765</v>
+        <v>767</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -7740,7 +7740,7 @@
         <v>2444</v>
       </c>
       <c r="M33">
-        <v>1615</v>
+        <v>1621</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -7781,7 +7781,7 @@
         <v>703</v>
       </c>
       <c r="M34">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -7822,7 +7822,7 @@
         <v>322</v>
       </c>
       <c r="M35">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -7863,7 +7863,7 @@
         <v>1425</v>
       </c>
       <c r="M36">
-        <v>927</v>
+        <v>931</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7904,7 +7904,7 @@
         <v>2337</v>
       </c>
       <c r="M37">
-        <v>1443</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -7945,7 +7945,7 @@
         <v>134</v>
       </c>
       <c r="M38">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -8068,7 +8068,7 @@
         <v>362</v>
       </c>
       <c r="M41">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -8109,7 +8109,7 @@
         <v>2494</v>
       </c>
       <c r="M42">
-        <v>1953</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -8150,7 +8150,7 @@
         <v>1461</v>
       </c>
       <c r="M43">
-        <v>711</v>
+        <v>714</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -8191,7 +8191,7 @@
         <v>972</v>
       </c>
       <c r="M44">
-        <v>615</v>
+        <v>616</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -8273,7 +8273,7 @@
         <v>301</v>
       </c>
       <c r="M46">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -8314,7 +8314,7 @@
         <v>940</v>
       </c>
       <c r="M47">
-        <v>600</v>
+        <v>603</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -8355,7 +8355,7 @@
         <v>2767</v>
       </c>
       <c r="M48">
-        <v>1701</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -8396,7 +8396,7 @@
         <v>1779</v>
       </c>
       <c r="M49">
-        <v>1100</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -8437,7 +8437,7 @@
         <v>1020</v>
       </c>
       <c r="M50">
-        <v>654</v>
+        <v>658</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -8478,7 +8478,7 @@
         <v>1445</v>
       </c>
       <c r="M51">
-        <v>940</v>
+        <v>943</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -8519,7 +8519,7 @@
         <v>1413</v>
       </c>
       <c r="M52">
-        <v>835</v>
+        <v>839</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -8560,7 +8560,7 @@
         <v>1756</v>
       </c>
       <c r="M53">
-        <v>1117</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -8601,7 +8601,7 @@
         <v>3832</v>
       </c>
       <c r="M54">
-        <v>2229</v>
+        <v>2237</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -8642,7 +8642,7 @@
         <v>1080</v>
       </c>
       <c r="M55">
-        <v>792</v>
+        <v>794</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -8683,7 +8683,7 @@
         <v>621</v>
       </c>
       <c r="M56">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -8724,7 +8724,7 @@
         <v>467</v>
       </c>
       <c r="M57">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -8847,7 +8847,7 @@
         <v>739</v>
       </c>
       <c r="M60">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="61" spans="1:13">
@@ -8929,7 +8929,7 @@
         <v>61</v>
       </c>
       <c r="M62">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="63" spans="1:13">
@@ -8970,7 +8970,7 @@
         <v>942</v>
       </c>
       <c r="M63">
-        <v>192</v>
+        <v>204</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -9011,7 +9011,7 @@
         <v>947</v>
       </c>
       <c r="M64">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -9052,7 +9052,7 @@
         <v>1385</v>
       </c>
       <c r="M65">
-        <v>861</v>
+        <v>863</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -9134,7 +9134,7 @@
         <v>1920</v>
       </c>
       <c r="M67">
-        <v>1216</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -9216,7 +9216,7 @@
         <v>473</v>
       </c>
       <c r="M69">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -9298,7 +9298,7 @@
         <v>346</v>
       </c>
       <c r="M71">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="72" spans="1:13">
@@ -9380,7 +9380,7 @@
         <v>1349</v>
       </c>
       <c r="M73">
-        <v>791</v>
+        <v>793</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -9421,7 +9421,7 @@
         <v>309</v>
       </c>
       <c r="M74">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:13">
@@ -9462,7 +9462,7 @@
         <v>427</v>
       </c>
       <c r="M75">
-        <v>275</v>
+        <v>279</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -9503,7 +9503,7 @@
         <v>3356</v>
       </c>
       <c r="M76">
-        <v>1883</v>
+        <v>1893</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -9544,7 +9544,7 @@
         <v>374</v>
       </c>
       <c r="M77">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -9585,7 +9585,7 @@
         <v>1583</v>
       </c>
       <c r="M78">
-        <v>731</v>
+        <v>735</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -9626,7 +9626,7 @@
         <v>2091</v>
       </c>
       <c r="M79">
-        <v>1109</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -9667,7 +9667,7 @@
         <v>470</v>
       </c>
       <c r="M80">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="81" spans="1:13">
@@ -9708,7 +9708,7 @@
         <v>187</v>
       </c>
       <c r="M81">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="82" spans="1:13">
@@ -9790,7 +9790,7 @@
         <v>1486</v>
       </c>
       <c r="M83">
-        <v>916</v>
+        <v>920</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -9831,7 +9831,7 @@
         <v>843</v>
       </c>
       <c r="M84">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="85" spans="1:13">
@@ -9872,7 +9872,7 @@
         <v>3396</v>
       </c>
       <c r="M85">
-        <v>2147</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -9913,7 +9913,7 @@
         <v>902</v>
       </c>
       <c r="M86">
-        <v>604</v>
+        <v>605</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -9995,7 +9995,7 @@
         <v>874</v>
       </c>
       <c r="M88">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -10036,7 +10036,7 @@
         <v>2036</v>
       </c>
       <c r="M89">
-        <v>1257</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -10077,7 +10077,7 @@
         <v>1089</v>
       </c>
       <c r="M90">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -10118,7 +10118,7 @@
         <v>968</v>
       </c>
       <c r="M91">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -10241,7 +10241,7 @@
         <v>2671</v>
       </c>
       <c r="M94">
-        <v>1730</v>
+        <v>1736</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -10282,7 +10282,7 @@
         <v>1241</v>
       </c>
       <c r="M95">
-        <v>761</v>
+        <v>766</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -10323,7 +10323,7 @@
         <v>1360</v>
       </c>
       <c r="M96">
-        <v>682</v>
+        <v>686</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -10364,7 +10364,7 @@
         <v>1719</v>
       </c>
       <c r="M97">
-        <v>949</v>
+        <v>954</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -10405,7 +10405,7 @@
         <v>1128</v>
       </c>
       <c r="M98">
-        <v>743</v>
+        <v>747</v>
       </c>
     </row>
     <row r="99" spans="1:13">
@@ -10446,7 +10446,7 @@
         <v>1505</v>
       </c>
       <c r="M99">
-        <v>980</v>
+        <v>983</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -10487,7 +10487,7 @@
         <v>277</v>
       </c>
       <c r="M100">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="101" spans="1:13">
@@ -10528,7 +10528,7 @@
         <v>104305</v>
       </c>
       <c r="M101">
-        <v>63178</v>
+        <v>63464</v>
       </c>
     </row>
   </sheetData>
@@ -11239,7 +11239,7 @@
         <v>293</v>
       </c>
       <c r="M3">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -11403,7 +11403,7 @@
         <v>21</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -11444,7 +11444,7 @@
         <v>319</v>
       </c>
       <c r="M8">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11485,7 +11485,7 @@
         <v>177</v>
       </c>
       <c r="M9">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -11567,7 +11567,7 @@
         <v>1920</v>
       </c>
       <c r="M11">
-        <v>1216</v>
+        <v>1221</v>
       </c>
     </row>
   </sheetData>
@@ -11674,7 +11674,7 @@
         <v>84</v>
       </c>
       <c r="M2">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -11920,7 +11920,7 @@
         <v>138</v>
       </c>
       <c r="M8">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -12043,7 +12043,7 @@
         <v>1015</v>
       </c>
       <c r="M11">
-        <v>765</v>
+        <v>767</v>
       </c>
     </row>
   </sheetData>
@@ -12314,7 +12314,7 @@
         <v>6</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -12519,7 +12519,7 @@
         <v>843</v>
       </c>
       <c r="M11">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -12667,7 +12667,7 @@
         <v>137</v>
       </c>
       <c r="M3">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -12872,7 +12872,7 @@
         <v>233</v>
       </c>
       <c r="M8">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -12995,7 +12995,7 @@
         <v>1385</v>
       </c>
       <c r="M11">
-        <v>861</v>
+        <v>863</v>
       </c>
     </row>
   </sheetData>
@@ -13418,7 +13418,7 @@
         <v>814</v>
       </c>
       <c r="M10">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13459,7 +13459,7 @@
         <v>1242</v>
       </c>
       <c r="M11">
-        <v>698</v>
+        <v>701</v>
       </c>
     </row>
   </sheetData>
@@ -13607,7 +13607,7 @@
         <v>294</v>
       </c>
       <c r="M3">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -13648,7 +13648,7 @@
         <v>16</v>
       </c>
       <c r="M4">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -13689,7 +13689,7 @@
         <v>171</v>
       </c>
       <c r="M5">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13812,7 +13812,7 @@
         <v>418</v>
       </c>
       <c r="M8">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13894,7 +13894,7 @@
         <v>902</v>
       </c>
       <c r="M10">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13935,7 +13935,7 @@
         <v>2337</v>
       </c>
       <c r="M11">
-        <v>1443</v>
+        <v>1453</v>
       </c>
     </row>
   </sheetData>
@@ -14109,7 +14109,7 @@
         <v>1</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -14305,7 +14305,7 @@
         <v>12</v>
       </c>
       <c r="M9">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -14387,7 +14387,7 @@
         <v>346</v>
       </c>
       <c r="M11">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>
@@ -14789,7 +14789,7 @@
         <v>180</v>
       </c>
       <c r="M10">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -14830,7 +14830,7 @@
         <v>301</v>
       </c>
       <c r="M11">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -15180,7 +15180,7 @@
         <v>105</v>
       </c>
       <c r="M8">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -15303,7 +15303,7 @@
         <v>739</v>
       </c>
       <c r="M11">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>
@@ -15410,7 +15410,7 @@
         <v>244</v>
       </c>
       <c r="M2">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15451,7 +15451,7 @@
         <v>220</v>
       </c>
       <c r="M3">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -15533,7 +15533,7 @@
         <v>194</v>
       </c>
       <c r="M5">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -15738,7 +15738,7 @@
         <v>939</v>
       </c>
       <c r="M10">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15779,7 +15779,7 @@
         <v>2412</v>
       </c>
       <c r="M11">
-        <v>1388</v>
+        <v>1394</v>
       </c>
     </row>
   </sheetData>
@@ -15927,7 +15927,7 @@
         <v>43</v>
       </c>
       <c r="M3">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -16117,7 +16117,7 @@
         <v>225</v>
       </c>
       <c r="M8">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -16199,7 +16199,7 @@
         <v>544</v>
       </c>
       <c r="M10">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16240,7 +16240,7 @@
         <v>947</v>
       </c>
       <c r="M11">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
   </sheetData>
@@ -16853,6 +16853,9 @@
       <c r="L4">
         <v>6</v>
       </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
@@ -16892,7 +16895,7 @@
         <v>91</v>
       </c>
       <c r="M5">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -17009,7 +17012,7 @@
         <v>360</v>
       </c>
       <c r="M8">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17091,7 +17094,7 @@
         <v>1954</v>
       </c>
       <c r="M10">
-        <v>1236</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17132,7 +17135,7 @@
         <v>2671</v>
       </c>
       <c r="M11">
-        <v>1730</v>
+        <v>1736</v>
       </c>
     </row>
   </sheetData>
@@ -17239,7 +17242,7 @@
         <v>68</v>
       </c>
       <c r="M2">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -17479,7 +17482,7 @@
         <v>208</v>
       </c>
       <c r="M8">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17561,7 +17564,7 @@
         <v>2713</v>
       </c>
       <c r="M10">
-        <v>1483</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17602,7 +17605,7 @@
         <v>3356</v>
       </c>
       <c r="M11">
-        <v>1883</v>
+        <v>1893</v>
       </c>
     </row>
   </sheetData>
@@ -18426,7 +18429,7 @@
         <v>200</v>
       </c>
       <c r="M10">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -18467,7 +18470,7 @@
         <v>277</v>
       </c>
       <c r="M11">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -18615,7 +18618,7 @@
         <v>60</v>
       </c>
       <c r="M3">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -18817,7 +18820,7 @@
         <v>203</v>
       </c>
       <c r="M8">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -18940,7 +18943,7 @@
         <v>580</v>
       </c>
       <c r="M11">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -19149,7 +19152,7 @@
         <v>48</v>
       </c>
       <c r="M5">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -19333,7 +19336,7 @@
         <v>587</v>
       </c>
       <c r="M10">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19374,7 +19377,7 @@
         <v>746</v>
       </c>
       <c r="M11">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -19709,7 +19712,7 @@
         <v>163</v>
       </c>
       <c r="M8">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -19791,7 +19794,7 @@
         <v>1379</v>
       </c>
       <c r="M10">
-        <v>816</v>
+        <v>818</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19832,7 +19835,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>1100</v>
+        <v>1103</v>
       </c>
     </row>
   </sheetData>
@@ -20179,7 +20182,7 @@
         <v>324</v>
       </c>
       <c r="M8">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20261,7 +20264,7 @@
         <v>1107</v>
       </c>
       <c r="M10">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20302,7 +20305,7 @@
         <v>1719</v>
       </c>
       <c r="M11">
-        <v>949</v>
+        <v>954</v>
       </c>
     </row>
   </sheetData>
@@ -20684,7 +20687,7 @@
         <v>25</v>
       </c>
       <c r="M9">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -20725,7 +20728,7 @@
         <v>427</v>
       </c>
       <c r="M10">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20766,7 +20769,7 @@
         <v>727</v>
       </c>
       <c r="M11">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -20873,7 +20876,7 @@
         <v>65</v>
       </c>
       <c r="M2">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -21119,7 +21122,7 @@
         <v>182</v>
       </c>
       <c r="M8">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21242,7 +21245,7 @@
         <v>1080</v>
       </c>
       <c r="M11">
-        <v>792</v>
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -21592,7 +21595,7 @@
         <v>358</v>
       </c>
       <c r="M8">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21674,7 +21677,7 @@
         <v>2940</v>
       </c>
       <c r="M10">
-        <v>1687</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21715,7 +21718,7 @@
         <v>3832</v>
       </c>
       <c r="M11">
-        <v>2229</v>
+        <v>2237</v>
       </c>
     </row>
   </sheetData>
@@ -21822,7 +21825,7 @@
         <v>61</v>
       </c>
       <c r="M2">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -22065,7 +22068,7 @@
         <v>207</v>
       </c>
       <c r="M8">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22188,7 +22191,7 @@
         <v>1349</v>
       </c>
       <c r="M11">
-        <v>791</v>
+        <v>793</v>
       </c>
     </row>
   </sheetData>
@@ -22295,7 +22298,7 @@
         <v>370</v>
       </c>
       <c r="M2">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -22336,7 +22339,7 @@
         <v>465</v>
       </c>
       <c r="M3">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -22377,7 +22380,7 @@
         <v>20</v>
       </c>
       <c r="M4">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -22500,7 +22503,7 @@
         <v>21</v>
       </c>
       <c r="M7">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -22541,7 +22544,7 @@
         <v>639</v>
       </c>
       <c r="M8">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22623,7 +22626,7 @@
         <v>1271</v>
       </c>
       <c r="M10">
-        <v>757</v>
+        <v>759</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22664,7 +22667,7 @@
         <v>3362</v>
       </c>
       <c r="M11">
-        <v>2038</v>
+        <v>2048</v>
       </c>
     </row>
   </sheetData>
@@ -22812,7 +22815,7 @@
         <v>180</v>
       </c>
       <c r="M3">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -22894,7 +22897,7 @@
         <v>191</v>
       </c>
       <c r="M5">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -22976,7 +22979,7 @@
         <v>9</v>
       </c>
       <c r="M7">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -23099,7 +23102,7 @@
         <v>1127</v>
       </c>
       <c r="M10">
-        <v>571</v>
+        <v>575</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -23140,7 +23143,7 @@
         <v>2333</v>
       </c>
       <c r="M11">
-        <v>1311</v>
+        <v>1318</v>
       </c>
     </row>
   </sheetData>
@@ -23845,7 +23848,7 @@
         <v>7</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -24032,7 +24035,7 @@
         <v>385</v>
       </c>
       <c r="M11">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -24139,7 +24142,7 @@
         <v>58</v>
       </c>
       <c r="M2">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -24499,7 +24502,7 @@
         <v>972</v>
       </c>
       <c r="M11">
-        <v>615</v>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -24606,7 +24609,7 @@
         <v>187</v>
       </c>
       <c r="M2">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -24852,7 +24855,7 @@
         <v>498</v>
       </c>
       <c r="M8">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24893,7 +24896,7 @@
         <v>190</v>
       </c>
       <c r="M9">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -24934,7 +24937,7 @@
         <v>1167</v>
       </c>
       <c r="M10">
-        <v>956</v>
+        <v>960</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24975,7 +24978,7 @@
         <v>2494</v>
       </c>
       <c r="M11">
-        <v>1953</v>
+        <v>1962</v>
       </c>
     </row>
   </sheetData>
@@ -25123,7 +25126,7 @@
         <v>69</v>
       </c>
       <c r="M3">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -25310,7 +25313,7 @@
         <v>251</v>
       </c>
       <c r="M8">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -25392,7 +25395,7 @@
         <v>2032</v>
       </c>
       <c r="M10">
-        <v>1311</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25433,7 +25436,7 @@
         <v>2767</v>
       </c>
       <c r="M11">
-        <v>1701</v>
+        <v>1705</v>
       </c>
     </row>
   </sheetData>
@@ -25968,7 +25971,7 @@
         <v>72</v>
       </c>
       <c r="M2">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -26208,7 +26211,7 @@
         <v>227</v>
       </c>
       <c r="M8">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -26331,7 +26334,7 @@
         <v>782</v>
       </c>
       <c r="M11">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
   </sheetData>
@@ -26672,7 +26675,7 @@
         <v>69</v>
       </c>
       <c r="M8">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -26713,7 +26716,7 @@
         <v>28</v>
       </c>
       <c r="M9">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -26754,7 +26757,7 @@
         <v>169</v>
       </c>
       <c r="M10">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26795,7 +26798,7 @@
         <v>362</v>
       </c>
       <c r="M11">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -27145,7 +27148,7 @@
         <v>437</v>
       </c>
       <c r="M8">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -27186,7 +27189,7 @@
         <v>67</v>
       </c>
       <c r="M9">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -27227,7 +27230,7 @@
         <v>638</v>
       </c>
       <c r="M10">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -27268,7 +27271,7 @@
         <v>1425</v>
       </c>
       <c r="M11">
-        <v>927</v>
+        <v>931</v>
       </c>
     </row>
   </sheetData>
@@ -27471,7 +27474,7 @@
         <v>14</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -27684,7 +27687,7 @@
         <v>267</v>
       </c>
       <c r="M11">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -28034,7 +28037,7 @@
         <v>122</v>
       </c>
       <c r="M8">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -28116,7 +28119,7 @@
         <v>824</v>
       </c>
       <c r="M10">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28157,7 +28160,7 @@
         <v>1155</v>
       </c>
       <c r="M11">
-        <v>746</v>
+        <v>749</v>
       </c>
     </row>
   </sheetData>
@@ -28550,7 +28553,7 @@
         <v>660</v>
       </c>
       <c r="M10">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28591,7 +28594,7 @@
         <v>902</v>
       </c>
       <c r="M11">
-        <v>604</v>
+        <v>605</v>
       </c>
     </row>
   </sheetData>
@@ -28739,7 +28742,7 @@
         <v>93</v>
       </c>
       <c r="M3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -29026,7 +29029,7 @@
         <v>976</v>
       </c>
       <c r="M10">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29067,7 +29070,7 @@
         <v>1583</v>
       </c>
       <c r="M11">
-        <v>731</v>
+        <v>735</v>
       </c>
     </row>
   </sheetData>
@@ -29746,7 +29749,7 @@
         <v>73</v>
       </c>
       <c r="M5">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -29951,7 +29954,7 @@
         <v>425</v>
       </c>
       <c r="M10">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29992,7 +29995,7 @@
         <v>813</v>
       </c>
       <c r="M11">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
   </sheetData>
@@ -30327,7 +30330,7 @@
         <v>113</v>
       </c>
       <c r="M8">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -30368,7 +30371,7 @@
         <v>16</v>
       </c>
       <c r="M9">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -30409,7 +30412,7 @@
         <v>307</v>
       </c>
       <c r="M10">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30450,7 +30453,7 @@
         <v>533</v>
       </c>
       <c r="M11">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>
@@ -30557,7 +30560,7 @@
         <v>78</v>
       </c>
       <c r="M2">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -30803,7 +30806,7 @@
         <v>251</v>
       </c>
       <c r="M8">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -30885,7 +30888,7 @@
         <v>762</v>
       </c>
       <c r="M10">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30926,7 +30929,7 @@
         <v>1360</v>
       </c>
       <c r="M11">
-        <v>682</v>
+        <v>686</v>
       </c>
     </row>
   </sheetData>
@@ -31270,7 +31273,7 @@
         <v>354</v>
       </c>
       <c r="M8">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -31311,7 +31314,7 @@
         <v>59</v>
       </c>
       <c r="M9">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -31352,7 +31355,7 @@
         <v>725</v>
       </c>
       <c r="M10">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31393,7 +31396,7 @@
         <v>1353</v>
       </c>
       <c r="M11">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
   </sheetData>
@@ -31541,7 +31544,7 @@
         <v>79</v>
       </c>
       <c r="M3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -31699,7 +31702,7 @@
         <v>7</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -31822,7 +31825,7 @@
         <v>813</v>
       </c>
       <c r="M10">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31863,7 +31866,7 @@
         <v>1445</v>
       </c>
       <c r="M11">
-        <v>940</v>
+        <v>943</v>
       </c>
     </row>
   </sheetData>
@@ -32093,7 +32096,7 @@
         <v>124</v>
       </c>
       <c r="M5">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -32175,7 +32178,7 @@
         <v>8</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -32216,7 +32219,7 @@
         <v>288</v>
       </c>
       <c r="M8">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -32298,7 +32301,7 @@
         <v>730</v>
       </c>
       <c r="M10">
-        <v>433</v>
+        <v>436</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32339,7 +32342,7 @@
         <v>1697</v>
       </c>
       <c r="M11">
-        <v>1018</v>
+        <v>1024</v>
       </c>
     </row>
   </sheetData>
@@ -32569,7 +32572,7 @@
         <v>40</v>
       </c>
       <c r="M5">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -32692,7 +32695,7 @@
         <v>250</v>
       </c>
       <c r="M8">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -32815,7 +32818,7 @@
         <v>968</v>
       </c>
       <c r="M11">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -33114,7 +33117,7 @@
         <v>28</v>
       </c>
       <c r="M8">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -33237,7 +33240,7 @@
         <v>277</v>
       </c>
       <c r="M11">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>
@@ -33344,7 +33347,7 @@
         <v>56</v>
       </c>
       <c r="M2">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -33578,7 +33581,7 @@
         <v>192</v>
       </c>
       <c r="M8">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -33619,7 +33622,7 @@
         <v>32</v>
       </c>
       <c r="M9">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -33660,7 +33663,7 @@
         <v>553</v>
       </c>
       <c r="M10">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33701,7 +33704,7 @@
         <v>940</v>
       </c>
       <c r="M11">
-        <v>600</v>
+        <v>603</v>
       </c>
     </row>
   </sheetData>
@@ -34054,7 +34057,7 @@
         <v>294</v>
       </c>
       <c r="M8">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -34095,7 +34098,7 @@
         <v>62</v>
       </c>
       <c r="M9">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -34177,7 +34180,7 @@
         <v>1089</v>
       </c>
       <c r="M11">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>
@@ -34325,7 +34328,7 @@
         <v>28</v>
       </c>
       <c r="M3">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -34597,7 +34600,7 @@
         <v>750</v>
       </c>
       <c r="M10">
-        <v>473</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34638,7 +34641,7 @@
         <v>1020</v>
       </c>
       <c r="M11">
-        <v>654</v>
+        <v>658</v>
       </c>
     </row>
   </sheetData>
@@ -35455,7 +35458,7 @@
         <v>185</v>
       </c>
       <c r="M8">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -35578,7 +35581,7 @@
         <v>642</v>
       </c>
       <c r="M11">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>
@@ -35808,7 +35811,7 @@
         <v>136</v>
       </c>
       <c r="M5">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -35928,7 +35931,7 @@
         <v>181</v>
       </c>
       <c r="M8">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -35969,7 +35972,7 @@
         <v>82</v>
       </c>
       <c r="M9">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -36010,7 +36013,7 @@
         <v>1425</v>
       </c>
       <c r="M10">
-        <v>901</v>
+        <v>902</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36051,7 +36054,7 @@
         <v>2036</v>
       </c>
       <c r="M11">
-        <v>1257</v>
+        <v>1263</v>
       </c>
     </row>
   </sheetData>
@@ -36158,7 +36161,7 @@
         <v>50</v>
       </c>
       <c r="M2">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -36199,7 +36202,7 @@
         <v>47</v>
       </c>
       <c r="M3">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -36483,7 +36486,7 @@
         <v>133</v>
       </c>
       <c r="M10">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36524,7 +36527,7 @@
         <v>374</v>
       </c>
       <c r="M11">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -36672,7 +36675,7 @@
         <v>4</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -36943,7 +36946,7 @@
         <v>621</v>
       </c>
       <c r="M11">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -37050,7 +37053,7 @@
         <v>17</v>
       </c>
       <c r="M2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -37152,7 +37155,7 @@
         <v>19</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -37389,7 +37392,7 @@
         <v>266</v>
       </c>
       <c r="M11">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -37824,7 +37827,7 @@
         <v>533</v>
       </c>
       <c r="M10">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -37865,7 +37868,7 @@
         <v>928</v>
       </c>
       <c r="M11">
-        <v>524</v>
+        <v>527</v>
       </c>
     </row>
   </sheetData>
@@ -38643,7 +38646,7 @@
         <v>189</v>
       </c>
       <c r="M8">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -38725,7 +38728,7 @@
         <v>1037</v>
       </c>
       <c r="M10">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38766,7 +38769,7 @@
         <v>1461</v>
       </c>
       <c r="M11">
-        <v>711</v>
+        <v>714</v>
       </c>
     </row>
   </sheetData>
@@ -38981,7 +38984,7 @@
         <v>8</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -39206,7 +39209,7 @@
         <v>128</v>
       </c>
       <c r="M11">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -39620,7 +39623,7 @@
         <v>408</v>
       </c>
       <c r="M10">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -39661,7 +39664,7 @@
         <v>597</v>
       </c>
       <c r="M11">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -39809,7 +39812,7 @@
         <v>17</v>
       </c>
       <c r="M3">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -39960,7 +39963,7 @@
         <v>30</v>
       </c>
       <c r="M8">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -40001,7 +40004,7 @@
         <v>35</v>
       </c>
       <c r="M9">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -40083,7 +40086,7 @@
         <v>470</v>
       </c>
       <c r="M11">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -40313,7 +40316,7 @@
         <v>52</v>
       </c>
       <c r="M5">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -40556,7 +40559,7 @@
         <v>703</v>
       </c>
       <c r="M11">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -40947,7 +40950,7 @@
         <v>90</v>
       </c>
       <c r="M9">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -40988,7 +40991,7 @@
         <v>1041</v>
       </c>
       <c r="M10">
-        <v>717</v>
+        <v>718</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -41029,7 +41032,7 @@
         <v>1779</v>
       </c>
       <c r="M11">
-        <v>1196</v>
+        <v>1198</v>
       </c>
     </row>
   </sheetData>
@@ -41174,7 +41177,7 @@
         <v>6</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -41442,7 +41445,7 @@
         <v>322</v>
       </c>
       <c r="M11">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -42616,7 +42619,7 @@
         <v>154</v>
       </c>
       <c r="M8">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -42698,7 +42701,7 @@
         <v>791</v>
       </c>
       <c r="M10">
-        <v>526</v>
+        <v>529</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -42739,7 +42742,7 @@
         <v>1128</v>
       </c>
       <c r="M11">
-        <v>743</v>
+        <v>747</v>
       </c>
     </row>
   </sheetData>
@@ -45414,7 +45417,7 @@
         <v>145</v>
       </c>
       <c r="M2">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -45455,7 +45458,7 @@
         <v>142</v>
       </c>
       <c r="M3">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -45537,7 +45540,7 @@
         <v>80</v>
       </c>
       <c r="M5">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -45742,7 +45745,7 @@
         <v>683</v>
       </c>
       <c r="M10">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45783,7 +45786,7 @@
         <v>1413</v>
       </c>
       <c r="M11">
-        <v>835</v>
+        <v>839</v>
       </c>
     </row>
   </sheetData>
@@ -46955,7 +46958,7 @@
         <v>56</v>
       </c>
       <c r="M8">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -47078,7 +47081,7 @@
         <v>467</v>
       </c>
       <c r="M11">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -47431,7 +47434,7 @@
         <v>182</v>
       </c>
       <c r="M8">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -47513,7 +47516,7 @@
         <v>433</v>
       </c>
       <c r="M10">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -47554,7 +47557,7 @@
         <v>874</v>
       </c>
       <c r="M11">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
   </sheetData>
@@ -47926,7 +47929,7 @@
         <v>264</v>
       </c>
       <c r="M10">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -47967,7 +47970,7 @@
         <v>309</v>
       </c>
       <c r="M11">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -48725,7 +48728,7 @@
         <v>117</v>
       </c>
       <c r="M10">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -48766,7 +48769,7 @@
         <v>187</v>
       </c>
       <c r="M11">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -49123,7 +49126,7 @@
         <v>93</v>
       </c>
       <c r="M10">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -49164,7 +49167,7 @@
         <v>134</v>
       </c>
       <c r="M11">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -49563,7 +49566,7 @@
         <v>253</v>
       </c>
       <c r="M10">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -49604,7 +49607,7 @@
         <v>414</v>
       </c>
       <c r="M11">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>